<commit_message>
feat(catalog): refresh shop dataset details
</commit_message>
<xml_diff>
--- a/docs/source/Dataset Shop Niuva/Niuva_Tokopedia_Products.xlsx
+++ b/docs/source/Dataset Shop Niuva/Niuva_Tokopedia_Products.xlsx
@@ -9,14 +9,16 @@
   <sheets>
     <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Variants" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Images" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Metadata" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Failures" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Details" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Images" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Metadata" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Failures" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products'!$A$1:$AU$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products'!$A$1:$AX$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Variants'!$A$1:$AI$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Images'!$A$1:$N$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Details'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Images'!$A$1:$N$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU9"/>
+  <dimension ref="A1:AX9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -476,18 +478,21 @@
     <col width="19" customWidth="1" min="33" max="33"/>
     <col width="50" customWidth="1" min="34" max="34"/>
     <col width="50" customWidth="1" min="35" max="35"/>
-    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
     <col width="50" customWidth="1" min="37" max="37"/>
     <col width="50" customWidth="1" min="38" max="38"/>
-    <col width="50" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
     <col width="50" customWidth="1" min="40" max="40"/>
     <col width="50" customWidth="1" min="41" max="41"/>
-    <col width="17" customWidth="1" min="42" max="42"/>
-    <col width="18" customWidth="1" min="43" max="43"/>
-    <col width="15" customWidth="1" min="44" max="44"/>
-    <col width="27" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="50" customWidth="1" min="42" max="42"/>
+    <col width="50" customWidth="1" min="43" max="43"/>
+    <col width="50" customWidth="1" min="44" max="44"/>
+    <col width="17" customWidth="1" min="45" max="45"/>
+    <col width="18" customWidth="1" min="46" max="46"/>
+    <col width="15" customWidth="1" min="47" max="47"/>
+    <col width="27" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,65 +668,80 @@
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
+          <t>detail_produk_lengkap</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>jumlah_bagian_detail</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>detail_produk_json</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
           <t>foto_utama_url</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>jumlah_foto</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>semua_foto_url_json</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>foto_utama_lokal</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>detail_items_json</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>variant_axes_json</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>detail_varian_json</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>halaman_listing</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>sumber_discovery</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>sumber_detail</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>diambil_pada</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>error</t>
         </is>
@@ -848,58 +868,82 @@
 - Ketika menerima paket, mohon rekam proses saat membuka paket</t>
         </is>
       </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=svD%2FMCbTAPMm2sw3axtTVj4uNsk%3D&amp;x-signature-webp=UiNX8Pb8pX4wBN4ZqxAXqh%2BYC4c%3D</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk Merchandise lucu berbasis 3D print!
+*** DETAIL PRODUK ***
+Material: PLA, Multicolor Print
+Size: 8 cm
+*** WAKTU PRODUKSI ***
+Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.
+~2–3 hari
+*** TERMS &amp; CONDITION ***
+- Refund tidak akan diterima apabila tidak ada video unboxing
+*** NOTE ***
+- Ketika menerima paket, mohon rekam proses saat membuka paket</t>
         </is>
       </c>
       <c r="AJ2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk Merchandise lucu berbasis 3D print!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk Merchandise lucu berbasis 3D print!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material: PLA, Multicolor Print\nSize: 8 cm", "lines": ["Material: PLA, Multicolor Print", "Size: 8 cm"], "bullets": []}, {"section_no": 3, "title": "WAKTU PRODUKSI", "text": "Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.\n~2–3 hari", "lines": ["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.", "~2–3 hari"], "bullets": []}, {"section_no": 4, "title": "TERMS &amp; CONDITION", "text": "- Refund tidak akan diterima apabila tidak ada video unboxing", "lines": ["- Refund tidak akan diterima apabila tidak ada video unboxing"], "bullets": ["Refund tidak akan diterima apabila tidak ada video unboxing"]}, {"section_no": 5, "title": "NOTE", "text": "- Ketika menerima paket, mohon rekam proses saat membuka paket", "lines": ["- Ketika menerima paket, mohon rekam proses saat membuka paket"], "bullets": ["Ketika menerima paket, mohon rekam proses saat membuka paket"]}]</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=4UISL%2FYJboBGuHt6v1SbO9Ryzwk%3D&amp;x-signature-webp=Jo2zBlT%2BgGlMuyjqqgYIkNt3UyA%3D</t>
+        </is>
+      </c>
+      <c r="AM2" t="n">
         <v>2</v>
       </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=svD%2FMCbTAPMm2sw3axtTVj4uNsk%3D&amp;x-signature-webp=UiNX8Pb8pX4wBN4ZqxAXqh%2BYC4c%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=MkefKNp5%2B1oQyUlL6iDIw%2FA%2FDGo%3D&amp;x-signature-webp=OVc29sBMOGQ%2FvVZ6zaQfDfonGkw%3D"]</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=4UISL%2FYJboBGuHt6v1SbO9Ryzwk%3D&amp;x-signature-webp=Jo2zBlT%2BgGlMuyjqqgYIkNt3UyA%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=XsGpxpSDGKqY5l2EYJZ7b2Qgeik%3D&amp;x-signature-webp=usEfoIBSW4MdqQdPseXbIMLLmow%3D"]</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
         <is>
           <t>Niuva_Product_Images\103726663896\gallery_001.jpg</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Gantungan Kunci"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AP2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AS2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT2" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:18:53+07:00</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:19+07:00</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1047,64 +1091,111 @@
 - Warna dilakukan secara manual menggunakan cat akrilik
 - Ketika menerima paket, mohon rekam proses saat membuka paket
 *** PRE ORDER CUSTOM ORDER ***
-- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan 
+- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan
 - Untuk pesanan custom customer WAJIB chat admin terlebih dahulu
 - Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
 - Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
         </is>
       </c>
-      <c r="AI3" s="2" t="inlineStr">
-        <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=2WvRYF4O2pDZ9vH2v9pFsbkwT48%3D&amp;x-signature-webp=oSOAwZPGCrxm8Nu4vSNrOJ5eAVA%3D</t>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+*** DETAIL PRODUK ***
+Variasi Figur Full-Color (Paint)
+Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 15 cm, 12 cm
+Variasi Figur Single Color
+Material: PLA, Single Color Print
+Size: 15 cm, 12 cm
+Variasi Lego Full-Color (Paint)
+Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 12 cm, 8 cm
+Variasi Lego Full-Color (MultiColor Print)
+Material: PLA, Multi-Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 12 cm, 8 cm
+Variasi Lego Single Color
+Material: PLA, Single Color Print
+Size: 12 cm, 8 cm
+*** WAKTU PRODUKSI ***
+Estimasi penyelesaian mengikuti durasi printing, custom paint job, dan kondisi antrian produksi.
+~6–7 hari
+*** TERMS &amp; CONDITION ***
+- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi
+- Finishing menggunakan hand painting
+- Refund tidak akan diterima apabila tidak ada video unboxing
+*** NOTE ***
+- Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket
+*** PRE ORDER CUSTOM ORDER ***
+- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan
+- Untuk pesanan custom customer WAJIB chat admin terlebih dahulu
+- Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
+- Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
         </is>
       </c>
       <c r="AJ3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Variasi Figur Full-Color (Paint)\nMaterial: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish\nSize: 15 cm, 12 cm\nVariasi Figur Single Color\nMaterial: PLA, Single Color Print\nSize: 15 cm, 12 cm\nVariasi Lego Full-Color (Paint)\nMaterial: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish\nSize: 12 cm, 8 cm\nVariasi Lego Full-Color (MultiColor Print)\nMaterial: PLA, Multi-Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish\nSize: 12 cm, 8 cm\nVariasi Lego Single Color\nMaterial: PLA, Single Color Print\nSize: 12 cm, 8 cm", "lines": ["Variasi Figur Full-Color (Paint)", "Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 15 cm, 12 cm", "Variasi Figur Single Color", "Material: PLA, Single Color Print", "Size: 15 cm, 12 cm", "Variasi Lego Full-Color (Paint)", "Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 12 cm, 8 cm", "Variasi Lego Full-Color (MultiColor Print)", "Material: PLA, Multi-Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 12 cm, 8 cm", "Variasi Lego Single Color", "Material: PLA, Single Color Print", "Size: 12 cm, 8 cm"], "bullets": []}, {"section_no": 3, "title": "WAKTU PRODUKSI", "text": "Estimasi penyelesaian mengikuti durasi printing, custom paint job, dan kondisi antrian produksi.\n~6–7 hari", "lines": ["Estimasi penyelesaian mengikuti durasi printing, custom paint job, dan kondisi antrian produksi.", "~6–7 hari"], "bullets": []}, {"section_no": 4, "title": "TERMS &amp; CONDITION", "text": "- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi\n- Finishing menggunakan hand painting\n- Refund tidak akan diterima apabila tidak ada video unboxing", "lines": ["- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi", "- Finishing menggunakan hand painting", "- Refund tidak akan diterima apabila tidak ada video unboxing"], "bullets": ["Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi", "Finishing menggunakan hand painting", "Refund tidak akan diterima apabila tidak ada video unboxing"]}, {"section_no": 5, "title": "NOTE", "text": "- Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)\n- Maksimal revisi adalah sebelum masuk masa cetak\n- Warna dilakukan secara manual menggunakan cat akrilik\n- Ketika menerima paket, mohon rekam proses saat membuka paket", "lines": ["- Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket"], "bullets": ["Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket"]}, {"section_no": 6, "title": "PRE ORDER CUSTOM ORDER", "text": "- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan\n- Untuk pesanan custom customer WAJIB chat admin terlebih dahulu\n- Pembayaran full 3 hari sebelum delivery (tidak ada deposit)\n- Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.", "lines": ["- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan", "- Untuk pesanan custom customer WAJIB chat admin terlebih dahulu", "- Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "- Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."], "bullets": ["Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan", "Untuk pesanan custom customer WAJIB chat admin terlebih dahulu", "Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."]}]</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=lVd4XUDpWS9eRMEqkfo%2BqooJq74%3D&amp;x-signature-webp=pp2yEsiGGIIvLKueQb1pY214YQU%3D</t>
+        </is>
+      </c>
+      <c r="AM3" t="n">
         <v>5</v>
       </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>["https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=2WvRYF4O2pDZ9vH2v9pFsbkwT48%3D&amp;x-signature-webp=oSOAwZPGCrxm8Nu4vSNrOJ5eAVA%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=WifDo1nzytofLdD5KU9pC0YX9XM%3D&amp;x-signature-webp=OyHmfon9RRjJgo6DUeLWei6u8KM%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=ExrUTK1UrT3PT1vCvxLDUQiSVpE%3D&amp;x-signature-webp=3dFzitryP31qFGQe1oMbcGzPNdA%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=3yfqcRPVECTQmgx6ChjVxk4UyL4%3D&amp;x-signature-webp=%2FDhE3JoMTuPEinrSTr%2BeR2ViDg4%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=9h08J1k%2By7jEMSAN0j4xvKF64qo%3D&amp;x-signature-webp=a%2FvWKMkIZ0htfkAGWv2ncSirE1g%3D"]</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=lVd4XUDpWS9eRMEqkfo%2BqooJq74%3D&amp;x-signature-webp=pp2yEsiGGIIvLKueQb1pY214YQU%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=KdpLa3GULJtv9AjRZatL6whc7ZI%3D&amp;x-signature-webp=URFFCPLSgZ8vTlDuGkIqMN7ETHE%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=qMIMIQ%2Bo9Mgb3pJUpi5eIuskNms%3D&amp;x-signature-webp=6nXxcwwjugD6xF1kR0NQuopW1Ls%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=TN%2BmsynoafUSezIdHeIhIui9cX4%3D&amp;x-signature-webp=FXNOEUSt7bnwZgoN%2B3Upw5j%2BeWM%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=pCHyfVTtO2d%2FYQejpL4P3G4QSe0%3D&amp;x-signature-webp=7gu5N1oS%2FBIoRszbJ%2B3OyeRzuD8%3D"]</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
         <is>
           <t>Niuva_Product_Images\103726333343\gallery_001.jpg</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AP3" t="inlineStr">
         <is>
           <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Bantal &amp; Boneka"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
         </is>
       </c>
-      <c r="AN3" t="inlineStr">
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>[{"name": "wisuda custom", "identifier": "", "options": [{"option_id": "3", "value": "Figur Custom Face", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}, {"option_id": "4", "value": "Figur Painted", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}, {"option_id": "5", "value": "Figur Single Color", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}, {"option_id": "6", "value": "Lego Painted", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}, {"option_id": "7", "value": "Lego Multicolor", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}, {"option_id": "8", "value": "Lego Single Color", "hex_color": "", "stock": 2, "picture_url": "", "picture_url_100": ""}]}, {"name": "ukuran", "identifier": "", "options": [{"option_id": "9", "value": "15 cm", "hex_color": "", "stock": 0, "picture_url": "", "picture_url_100": ""}, {"option_id": "10", "value": "12 cm", "hex_color": "", "stock": 0, "picture_url": "", "picture_url_100": ""}, {"option_id": "11", "value": "8 cm", "hex_color": "", "stock": 0, "picture_url": "", "picture_url_100": ""}]}]</t>
         </is>
       </c>
-      <c r="AO3" t="inlineStr">
+      <c r="AR3" t="inlineStr">
         <is>
           <t>[{"product_id": "103726333343", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890", "price": 95000, "price_payload": 95000, "price_fmt": "Rp95.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3", "9"], "option_names": ["Figur Custom Face", "15 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333344", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663836426", "price": 75000, "price_payload": 75000, "price_fmt": "Rp75.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3", "10"], "option_names": ["Figur Custom Face", "12 cm"], "option_names_raw": ["Figur Custom Face", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333345", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Painted, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Painted, 15 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663901962", "price": 85000, "price_payload": 85000, "price_fmt": "Rp85.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4", "9"], "option_names": ["Figur Painted", "15 cm"], "option_names_raw": ["Figur Painted", "15 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333346", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Painted, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Painted, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663967498", "price": 65000, "price_payload": 65000, "price_fmt": "Rp65.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4", "10"], "option_names": ["Figur Painted", "12 cm"], "option_names_raw": ["Figur Painted", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333347", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Single Color, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Single Color, 15 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664033034", "price": 65000, "price_payload": 65000, "price_fmt": "Rp65.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["5", "9"], "option_names": ["Figur Single Color", "15 cm"], "option_names_raw": ["Figur Single Color", "15 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333348", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Single Color, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Single Color, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664098570", "price": 45000, "price_payload": 45000, "price_fmt": "Rp45.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["5", "10"], "option_names": ["Figur Single Color", "12 cm"], "option_names_raw": ["Figur Single Color", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333349", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Painted, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Painted, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664164106", "price": 80000, "price_payload": 80000, "price_fmt": "Rp80.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["6", "10"], "option_names": ["Lego Painted", "12 cm"], "option_names_raw": ["Lego Painted", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333350", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Painted, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Painted, 8 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664229642", "price": 60000, "price_payload": 60000, "price_fmt": "Rp60.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["6", "11"], "option_names": ["Lego Painted", "8 cm"], "option_names_raw": ["Lego Painted", "8 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333351", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Multicolor, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Multicolor, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664295178", "price": 150000, "price_payload": 150000, "price_fmt": "Rp150.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["7", "10"], "option_names": ["Lego Multicolor", "12 cm"], "option_names_raw": ["Lego Multicolor", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333352", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Multicolor, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Multicolor, 8 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664360714", "price": 80000, "price_payload": 80000, "price_fmt": "Rp80.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["7", "11"], "option_names": ["Lego Multicolor", "8 cm"], "option_names_raw": ["Lego Multicolor", "8 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333353", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Single Color, 12 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Single Color, 12 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664426250", "price": 55000, "price_payload": 55000, "price_fmt": "Rp55.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["8", "10"], "option_names": ["Lego Single Color", "12 cm"], "option_names_raw": ["Lego Single Color", "12 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103726333354", "product_name": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Single Color, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Lego Single Color, 8 cm", "product_url": "https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528664491786", "price": 35000, "price_payload": 35000, "price_fmt": "Rp35.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["8", "11"], "option_names": ["Lego Single Color", "8 cm"], "option_names_raw": ["Lego Single Color", "8 cm"], "stock": 1, "is_buyable": true, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Figur Custom Face, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["3", "11"], "option_names": ["Figur Custom Face", "8 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Figur Painted, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["4", "11"], "option_names": ["Figur Painted", "8 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Figur Single Color, 8 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["5", "11"], "option_names": ["Figur Single Color", "8 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Lego Painted, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["6", "9"], "option_names": ["Lego Painted", "15 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Lego Multicolor, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["7", "9"], "option_names": ["Lego Multicolor", "15 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}, {"product_id": "-9223371933128442465", "product_name": "Wisuda Custom 3D Print - Lego Single Color, 15 cm", "product_name_raw": "Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus - Figur Custom Face, 15 cm", "product_url": null, "price": null, "price_payload": 95000, "price_fmt": "", "original_price": null, "slash_price_fmt": "", "discount_percentage": null, "option_ids": ["8", "9"], "option_names": ["Lego Single Color", "15 cm"], "option_names_raw": ["Figur Custom Face", "15 cm"], "stock": 0, "is_buyable": false, "minimum_order": 1, "maximum_order": 1, "stock_message": "Stok terakhir, beli sekarang!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/70f78c7827e64a44ae2300b7a55eb96f~.jpeg", "is_placeholder": true, "status": "PLACEHOLDER_TOKOPEDIA"}]</t>
         </is>
       </c>
-      <c r="AP3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ3" t="inlineStr">
+      <c r="AS3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT3" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:18:55+07:00</t>
-        </is>
-      </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:24+07:00</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1229,350 +1320,7 @@
 Komplain tanpa bukti video tidak dapat diproses</t>
         </is>
       </c>
-      <c r="AI4" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=tqAdXHjGXCOUSW3eaHZLt9qaAvU%3D&amp;x-signature-webp=5HsayE8Hv1J7LrIcmqUE1TWGhpA%3D</t>
-        </is>
-      </c>
-      <c r="AJ4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=tqAdXHjGXCOUSW3eaHZLt9qaAvU%3D&amp;x-signature-webp=5HsayE8Hv1J7LrIcmqUE1TWGhpA%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=R8SMoLrgf6%2BEa6d9u6DfW8M82PM%3D&amp;x-signature-webp=zfwyhXJ3RrxAI%2BsPAPogPjJCG1k%3D"]</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>Niuva_Product_Images\103474501379\gallery_001.jpg</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Figure Set"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AP4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ4" t="inlineStr">
-        <is>
-          <t>apollo_cache</t>
-        </is>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>apollo_cache</t>
-        </is>
-      </c>
-      <c r="AS4" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:18:58+07:00</t>
-        </is>
-      </c>
-      <c r="AT4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>103343689816</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>7494627384206133002</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>35200</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>35200</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n">
-        <v>30400</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>35200</v>
-      </c>
-      <c r="K5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="n">
-        <v>3</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
-        <v>5</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Gantungan Kunci</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Perlengkapan Pesta &gt; Hadiah &gt; Gantungan Kunci</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Semua Etalase</t>
-        </is>
-      </c>
-      <c r="AE5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>KILOGRAM</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>1 Buah</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>NIUVA STUDIO – Jasa 3D print custom
-Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
-DETAIL PRODUK :
-Material : PLA
-Size: 8cm
-Layer height : 0.2mm
-Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
-        </is>
-      </c>
-      <c r="AI5" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=Hh%2Bu8u%2FUdoOjIoP%2Fd1fMcWARPfs%3D&amp;x-signature-webp=aL0aZwXndr8wLDsEIVpjPk5284E%3D</t>
-        </is>
-      </c>
-      <c r="AJ5" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=Hh%2Bu8u%2FUdoOjIoP%2Fd1fMcWARPfs%3D&amp;x-signature-webp=aL0aZwXndr8wLDsEIVpjPk5284E%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=0Hklwo%2BwJ0mQNelPLvc950PeWXU%3D&amp;x-signature-webp=BPq9W2FGcgi2edMK%2BfUTAgnlzlw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=8JLonBXZnCN8wAn3EjLeDlRilvw%3D&amp;x-signature-webp=PoDzEMvYgyuCCCzT2htgMymxQ4s%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=Mk6p9D7Q7BJ%2B2hiNdPqoQz5w4i0%3D&amp;x-signature-webp=0QRT5j6ABMvHZG20oa6F24scQFU%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=JJDsqmXPE785hYKZRffQtEi1x2k%3D&amp;x-signature-webp=JUneY87LJqx%2BfdAPeNPx65dblGA%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=iUujNWD9UkeWfjC69b6x%2BCe1eEk%3D&amp;x-signature-webp=U1COq%2F0RkmE%2F4r0NJz6ymhy7BtU%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=TZexh%2F1rHRKlwQX8vs5uyLZZSjk%3D&amp;x-signature-webp=v5ofvoUUvnl%2Bnj36PaO3CpfSQJc%3D"]</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>Niuva_Product_Images\103343689816\gallery_001.jpg</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Gantungan Kunci"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>[{"name": "gedung", "identifier": "", "options": [{"option_id": "2", "value": "TULT BIRU", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg"}, {"option_id": "3", "value": "BANDUNG TECHNO PARK", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg"}, {"option_id": "4", "value": "TULT ABU", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg"}]}]</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>[{"product_id": "103343689816", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT BIRU", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT BIRU", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922", "price": 35200, "price_payload": 35200, "price_fmt": "Rp35.200", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["TULT BIRU"], "option_names_raw": ["TULT BIRU"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343689817", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - BANDUNG TECHNO PARK", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - BANDUNG TECHNO PARK", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114440458", "price": 30400, "price_payload": 30400, "price_fmt": "Rp30.400", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["BANDUNG TECHNO PARK"], "option_names_raw": ["BANDUNG TECHNO PARK"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343689818", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT ABU", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT ABU", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114505994", "price": 30400, "price_payload": 30400, "price_fmt": "Rp30.400", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4"], "option_names": ["TULT ABU"], "option_names_raw": ["TULT ABU"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
-        </is>
-      </c>
-      <c r="AP5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>apollo_cache</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>apollo_cache</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:19:00+07:00</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>103343687481</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>7494627384206133002</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n">
-        <v>150000</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>150000</v>
-      </c>
-      <c r="K6" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Action Figure</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>Mainan &amp; Hobi &gt; Figure &gt; Action Figure</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>Semua Etalase</t>
-        </is>
-      </c>
-      <c r="AE6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>KILOGRAM</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>1 Buah</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>NIUVA STUDIO - Jasa 3D print custom
 Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
@@ -1586,173 +1334,181 @@
 Komplain tanpa bukti video tidak dapat diproses</t>
         </is>
       </c>
-      <c r="AI6" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=%2FFwwqWaNvZdwruwp%2BNJw%2BKF%2FuFs%3D&amp;x-signature-webp=AnZBI%2FTNDFGO9U8ZQixt6v%2B509A%3D</t>
-        </is>
-      </c>
-      <c r="AJ6" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK6" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=%2FFwwqWaNvZdwruwp%2BNJw%2BKF%2FuFs%3D&amp;x-signature-webp=AnZBI%2FTNDFGO9U8ZQixt6v%2B509A%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=wVnXi7THp5FtYJHyCRGrcOGx%2BFE%3D&amp;x-signature-webp=uSyuCSgr0q5cjstt9qa8ahm83PE%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=5R6bzPRXu2Py7FmejIIhIoFdnHw%3D&amp;x-signature-webp=wczkX6X%2F6xnpAqx1oGOT1c8eDVw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=6jxF%2B2%2FXpDO4pcoiX11r2pPSeuM%3D&amp;x-signature-webp=psK1x639Vjsc7E5Xi7nxIEh0oTQ%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=W3p2zPMK6d1mP5UHL4mOm3VD3aE%3D&amp;x-signature-webp=EntRhQ7rBqgEkexcjjvef8S1PsE%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=GTwlZXJxHoplnnkSDJ13D6QSVK8%3D&amp;x-signature-webp=yBj%2BGD9d43khH29f5rZQz%2Blf8VM%3D"]</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>Niuva_Product_Images\103343687481\gallery_001.jpg</t>
-        </is>
-      </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Action Figure"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
-        </is>
-      </c>
-      <c r="AN6" t="inlineStr">
-        <is>
-          <t>[{"name": "gender", "identifier": "", "options": [{"option_id": "2", "value": "PEREMPUAN", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg"}, {"option_id": "3", "value": "LAKI LAKI", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg"}]}]</t>
-        </is>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>[{"product_id": "103343687481", "product_name": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - PEREMPUAN", "product_name_raw": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - PEREMPUAN", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074", "price": 150000, "price_payload": 150000, "price_fmt": "Rp150.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["PEREMPUAN"], "option_names_raw": ["PEREMPUAN"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343687482", "product_name": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - LAKI LAKI", "product_name_raw": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - LAKI LAKI", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198969610", "price": 150000, "price_payload": 150000, "price_fmt": "Rp150.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["LAKI LAKI"], "option_names_raw": ["LAKI LAKI"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
-        </is>
-      </c>
-      <c r="AP6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ6" t="inlineStr">
+      <c r="AJ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO - Jasa 3D print custom\nNiuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO - Jasa 3D print custom", "Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material: PLA\nSize: 12cm\nLayer height : 0.2mm", "lines": ["Material: PLA", "Size: 12cm", "Layer height : 0.2mm"], "bullets": []}, {"section_no": 3, "title": "NOTES", "text": "- tulis fakultas di notes/chat yaa\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.\nKomplain tanpa bukti video tidak dapat diproses", "lines": ["- tulis fakultas di notes/chat yaa", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.", "Komplain tanpa bukti video tidak dapat diproses"], "bullets": ["tulis fakultas di notes/chat yaa"]}]</t>
+        </is>
+      </c>
+      <c r="AL4" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=j3QM%2Bnlx1YUB2%2Bd3r%2FYdkcPq%2Bjk%3D&amp;x-signature-webp=BDhDKtuKqO62qEOXTE8om5%2BGnTE%3D</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=j3QM%2Bnlx1YUB2%2Bd3r%2FYdkcPq%2Bjk%3D&amp;x-signature-webp=BDhDKtuKqO62qEOXTE8om5%2BGnTE%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=A%2BLggcWo1DNN4xASKtWrj6m1XZY%3D&amp;x-signature-webp=d%2F1P%2Fpi3DYifmMwjKTW7HYXJCz0%3D"]</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Niuva_Product_Images\103474501379\gallery_001.jpg</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Figure Set"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AS4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT4" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AU4" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:19:04+07:00</t>
-        </is>
-      </c>
-      <c r="AT6" t="inlineStr">
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:28+07:00</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>103342790916</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>103343689816</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>7494627384206133002</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441002762</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="K7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>35200</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>35200</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n">
+        <v>30400</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>35200</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
         <v>5</v>
       </c>
-      <c r="N7" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>5</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="inlineStr">
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>Baru</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>Gantungan Kunci</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Perlengkapan Pesta &gt; Hadiah &gt; Gantungan Kunci</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Semua Etalase</t>
         </is>
       </c>
-      <c r="AE7" t="n">
+      <c r="AE5" t="n">
         <v>0.2</v>
       </c>
-      <c r="AF7" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>KILOGRAM</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>1 Buah</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>NIUVA STUDIO – Jasa 3D print custom
 Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
@@ -1763,58 +1519,475 @@
 Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
         </is>
       </c>
-      <c r="AI7" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2B%2FqDYKSQU2iQY82D%2F04kwKtDrnA%3D&amp;x-signature-webp=U1W4UNKcuFeFrxUyFXoAk49zVdU%3D</t>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material : PLA
+Size: 8cm
+Layer height : 0.2mm
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="AJ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material : PLA\nSize: 8cm\nLayer height : 0.2mm\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses", "lines": ["Material : PLA", "Size: 8cm", "Layer height : 0.2mm", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses"], "bullets": []}]</t>
+        </is>
+      </c>
+      <c r="AL5" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=bSSq4nt%2B1%2BQjDqLw2xZ%2FF4DE6Z8%3D&amp;x-signature-webp=8n8x3kU2zcCyaMWhj70OApnJKJM%3D</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=bSSq4nt%2B1%2BQjDqLw2xZ%2FF4DE6Z8%3D&amp;x-signature-webp=8n8x3kU2zcCyaMWhj70OApnJKJM%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=Enc4sPipEhn9qLy%2BX4Hw4ZNBOO4%3D&amp;x-signature-webp=%2FiyRGB8bTXq3JFHOKx7XGzQlv9s%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=S0V9KaIXwAAUyiWNXU%2FzcTTewmg%3D&amp;x-signature-webp=%2BDyuTyDAvzVRTwIUnNFp5Sp2gAI%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=gjB3D6cjx7Uf7vIuqJNjUJz6Lao%3D&amp;x-signature-webp=olv1eG3Z6fgGkeHTVLVG9BJVsIg%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=KxW%2FEv%2FZPm5Tr6qsPRsaR8Hwd3o%3D&amp;x-signature-webp=X0pf3N4Ke%2BpPNRNy7mLKTp4Snh8%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=Z63dV%2BXuCj8ot1r1nJULWKqHUxg%3D&amp;x-signature-webp=ZOE2nrBkGzz8Pd81yQUSW4HGoxw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=avYJt9P47i7tQfeYBx3wb2qPwTw%3D&amp;x-signature-webp=gw6fCLHQeNrvT%2FtnjWPjbUsjnYY%3D"]</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Niuva_Product_Images\103343689816\gallery_001.jpg</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Gantungan Kunci"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>[{"name": "gedung", "identifier": "", "options": [{"option_id": "2", "value": "TULT BIRU", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg"}, {"option_id": "3", "value": "BANDUNG TECHNO PARK", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg"}, {"option_id": "4", "value": "TULT ABU", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg"}]}]</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>[{"product_id": "103343689816", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT BIRU", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT BIRU", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922", "price": 35200, "price_payload": 35200, "price_fmt": "Rp35.200", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["TULT BIRU"], "option_names_raw": ["TULT BIRU"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/e140811d00c343c3b00983a8d73258b2~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343689817", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - BANDUNG TECHNO PARK", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - BANDUNG TECHNO PARK", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114440458", "price": 30400, "price_payload": 30400, "price_fmt": "Rp30.400", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["BANDUNG TECHNO PARK"], "option_names_raw": ["BANDUNG TECHNO PARK"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/9b0225eaec684b00915445a816ff3992~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343689818", "product_name": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT ABU", "product_name_raw": "3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK) - TULT ABU", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114505994", "price": 30400, "price_payload": 30400, "price_fmt": "Rp30.400", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4"], "option_names": ["TULT ABU"], "option_names_raw": ["TULT ABU"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1bad1d2dc25c44f88797cc5dad2f220e~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
+        </is>
+      </c>
+      <c r="AS5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:33+07:00</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>103343687481</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>7494627384206133002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>5</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Action Figure</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Mainan &amp; Hobi &gt; Figure &gt; Action Figure</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Semua Etalase</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>KILOGRAM</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>1 Buah</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO - Jasa 3D print custom
+Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material: PLA
+Size: 12cm
+Layer height : 0.2mm
+NOTES :
+- tulis fakultas di notes/chat yaa
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.
+Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO - Jasa 3D print custom
+Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material: PLA
+Size: 12cm
+Layer height : 0.2mm
+NOTES :
+- tulis fakultas di notes/chat yaa
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.
+Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="AJ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO - Jasa 3D print custom\nNiuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO - Jasa 3D print custom", "Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material: PLA\nSize: 12cm\nLayer height : 0.2mm", "lines": ["Material: PLA", "Size: 12cm", "Layer height : 0.2mm"], "bullets": []}, {"section_no": 3, "title": "NOTES", "text": "- tulis fakultas di notes/chat yaa\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.\nKomplain tanpa bukti video tidak dapat diproses", "lines": ["- tulis fakultas di notes/chat yaa", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.", "Komplain tanpa bukti video tidak dapat diproses"], "bullets": ["tulis fakultas di notes/chat yaa"]}]</t>
+        </is>
+      </c>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=UHRS3L9fCzWRI5Mv8TgaUHFfO3E%3D&amp;x-signature-webp=jJ9GvtcNqj70tc60O1kw89b32%2Bw%3D</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=UHRS3L9fCzWRI5Mv8TgaUHFfO3E%3D&amp;x-signature-webp=jJ9GvtcNqj70tc60O1kw89b32%2Bw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=lZeu7C6aK4bjBLGWFDddFFeg%2BFE%3D&amp;x-signature-webp=gix3sHTEbgot1YYcvt94uit46iI%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=Bw6teuiMfsmK8NMVjTyt1GTactg%3D&amp;x-signature-webp=0LskqGPE25qB4cwFNGQRqhZ6taw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=EbWMLrqpMLGpORahKe1%2BLiUMzpQ%3D&amp;x-signature-webp=BOUrY8Dpq2ukJK3Gv3IRSrvaY6w%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=cUuAAydx2LaOua2pACovM4Niidc%3D&amp;x-signature-webp=B4Qu18bZe0QvxPAVUNzVpLn2oGw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=XmHZ2xT17HsceQ6arKyjq0e27cU%3D&amp;x-signature-webp=pzPaLXx6iWy2%2BbM1mwe4LrZI5wc%3D"]</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Niuva_Product_Images\103343687481\gallery_001.jpg</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Action Figure"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>[{"name": "gender", "identifier": "", "options": [{"option_id": "2", "value": "PEREMPUAN", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg"}, {"option_id": "3", "value": "LAKI LAKI", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg"}]}]</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>[{"product_id": "103343687481", "product_name": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - PEREMPUAN", "product_name_raw": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - PEREMPUAN", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074", "price": 150000, "price_payload": 150000, "price_fmt": "Rp150.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["PEREMPUAN"], "option_names_raw": ["PEREMPUAN"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/66488a928e8042519c6676d816cd6471~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103343687482", "product_name": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - LAKI LAKI", "product_name_raw": "3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas) - LAKI LAKI", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198969610", "price": 150000, "price_payload": 150000, "price_fmt": "Rp150.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["LAKI LAKI"], "option_names_raw": ["LAKI LAKI"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1754b3fc687d4f4b9dfdc746f39386bc~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
+        </is>
+      </c>
+      <c r="AS6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:36+07:00</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>103342790916</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7494627384206133002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441002762</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>5</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Gantungan Kunci</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Perlengkapan Pesta &gt; Hadiah &gt; Gantungan Kunci</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Semua Etalase</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>KILOGRAM</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>1 Buah</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material : PLA
+Size: 8cm
+Layer height : 0.2mm
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material : PLA
+Size: 8cm
+Layer height : 0.2mm
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
         </is>
       </c>
       <c r="AJ7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material : PLA\nSize: 8cm\nLayer height : 0.2mm\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses", "lines": ["Material : PLA", "Size: 8cm", "Layer height : 0.2mm", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses"], "bullets": []}]</t>
+        </is>
+      </c>
+      <c r="AL7" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=Tbv3SzY4pEdpnKY%2F%2FAHiLk2OUxo%3D&amp;x-signature-webp=x6%2FYKs%2B1jqrgT0fxT6dete4Neio%3D</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
         <v>12</v>
       </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2B%2FqDYKSQU2iQY82D%2F04kwKtDrnA%3D&amp;x-signature-webp=U1W4UNKcuFeFrxUyFXoAk49zVdU%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=PjEZtnYONb0GEoAfAIH4BEKa1lg%3D&amp;x-signature-webp=V6drDG7x0MudqCYfWkb5FTBs6SM%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=vEP1H1e%2FcdMFuq6I4S5Y%2B5JzSto%3D&amp;x-signature-webp=N1e4aj2k8HcihssYPJ477K%2BVwzA%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=0IuXjlHYaijpntTooGIdKoTJ474%3D&amp;x-signature-webp=M8En%2B13b4itIZiYzrQ8K4oI9HzQ%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=fpdtfLXoP6mS9U40r9oRGv8vuc0%3D&amp;x-signature-webp=YfGeB%2Byz4krOJda%2BG0Bs2QWH6Os%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2Bl1f32hH99dRDOxN%2B7XO2Hxry5k%3D&amp;x-signature-webp=MhmyDPKb1%2BrlA7ZX9lMVU3eqFJg%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=TyjJGpuCkRBmLsxJNKhmzePzXig%3D&amp;x-signature-webp=wgoxJaBlU6nC2l%2BI0F1dsFGh7zI%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=awJdlSl%2F1GQjHweRRXzILjHL1JI%3D&amp;x-signature-webp=ZI19cOWc%2FCtz4YnEnd2hOzYzJ0c%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=IPDcC%2Bg9IvVN708HG%2BlFs1HbqnU%3D&amp;x-signature-webp=kAJoLffigibljWjZ3gdDqmqngzw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=8MfAkc9zYs6C%2FiIBhPx3BpPJwsw%3D&amp;x-signature-webp=sCCJZWYd%2BEy79PXHgHq0UInRviw%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=BsdT094hOEdEVVoPIK0dtvIzIGg%3D&amp;x-signature-webp=P6979aJFlO5Wvbg5T5Tfq4t8eF0%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=rrUT5pVf05k8KerYH%2FilR0OnPH0%3D&amp;x-signature-webp=RTMh%2F%2BMnt%2Ff%2BCxf0DA3DzZ4ReLg%3D"]</t>
-        </is>
-      </c>
-      <c r="AL7" t="inlineStr">
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=Tbv3SzY4pEdpnKY%2F%2FAHiLk2OUxo%3D&amp;x-signature-webp=x6%2FYKs%2B1jqrgT0fxT6dete4Neio%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=NCgs4BPRULa9SVHE4XymMNM6gQ8%3D&amp;x-signature-webp=ck0EXTnn44e4OyL8z%2BZTYVixgHs%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=BMPKDGFuGiYnf6Ka%2FNYc8%2BZ5l9E%3D&amp;x-signature-webp=C1Tj%2FldGi9dN9a%2FVhgBRmIoNEBg%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=71x%2F%2BHY0Gc%2FMvDt0EcH4yMNk5T4%3D&amp;x-signature-webp=uY926%2FVTfX5Itg4rOIdR%2BVQIpIM%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=RBB33UQkJouuV3trfY8ZLAVEM4E%3D&amp;x-signature-webp=YPYb3jSntbW%2BK1PDNNPxVfTw4ww%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=4qN%2B2zzlw72Ly%2BzwEIvAp3X1nt0%3D&amp;x-signature-webp=JyNfnN3CzJgWJGn2c3EejbVQzgU%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=pz36nJZN%2FLELk8U5vRHRYeifCu8%3D&amp;x-signature-webp=wBbAZHUdxRT8lKa%2B4eVlOC9q6Z4%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=HtpS%2BJcNmXMU3cLWQorpBDxNA%2Bc%3D&amp;x-signature-webp=%2BcrXy0adH1s6DDunjvNXQtHo6V8%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=s3XpZJFXR2zBwZizMgnLKyrYWNw%3D&amp;x-signature-webp=IUbEhRgmlsIqC7y3F4eFSYZ0HMo%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=P1WWhj4g85KoTql%2BIF1uywv7ef0%3D&amp;x-signature-webp=UBhM50sYzZWs%2F0KGoN%2FyAWCboQY%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=bS0uKvQG9446EsvLtwNd6dwIBsI%3D&amp;x-signature-webp=41X68TO8cz8oodz8gu5TIW088T4%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=5sKpH73qCtr7ic7Tsob7iE1gpPM%3D&amp;x-signature-webp=6jzUOQ5ggjoEeD7P8glx4kZ%2F0ac%3D"]</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
         <is>
           <t>Niuva_Product_Images\103342790916\gallery_001.jpg</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr">
+      <c r="AP7" t="inlineStr">
         <is>
           <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Gantungan Kunci"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
         </is>
       </c>
-      <c r="AN7" t="inlineStr">
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>[{"name": "animal mascot", "identifier": "", "options": [{"option_id": "2", "value": "soang baju merah", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/5806fc2a7e6c448b87838e59e75f1929~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/5806fc2a7e6c448b87838e59e75f1929~.jpeg"}, {"option_id": "3", "value": "soang baju putih", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/01c44a71ca8d4f43999a6e8fa94f0724~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/01c44a71ca8d4f43999a6e8fa94f0724~.jpeg"}, {"option_id": "4", "value": "maung wisuda", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/17559de5f5f846daa12442c61d6f21c9~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/17559de5f5f846daa12442c61d6f21c9~.jpeg"}, {"option_id": "5", "value": "galih", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1e5c62974cfe4f06848cd22418272c87~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1e5c62974cfe4f06848cd22418272c87~.jpeg"}, {"option_id": "6", "value": "merak", "hex_color": "", "stock": 5, "picture_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/3de569aff3154f90840bf0a9ecfb4ff9~.jpeg.webp", "picture_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/3de569aff3154f90840bf0a9ecfb4ff9~.jpeg"}]}]</t>
         </is>
       </c>
-      <c r="AO7" t="inlineStr">
+      <c r="AR7" t="inlineStr">
         <is>
           <t>[{"product_id": "103342790916", "product_name": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - soang baju merah", "product_name_raw": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - soang baju merah", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441002762", "price": 20000, "price_payload": 20000, "price_fmt": "Rp20.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["soang baju merah"], "option_names_raw": ["soang baju merah"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/5806fc2a7e6c448b87838e59e75f1929~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/5806fc2a7e6c448b87838e59e75f1929~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103342790917", "product_name": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - soang baju putih", "product_name_raw": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - soang baju putih", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441068298", "price": 20000, "price_payload": 20000, "price_fmt": "Rp20.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["soang baju putih"], "option_names_raw": ["soang baju putih"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/01c44a71ca8d4f43999a6e8fa94f0724~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/01c44a71ca8d4f43999a6e8fa94f0724~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103342790918", "product_name": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - maung wisuda", "product_name_raw": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - maung wisuda", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441133834", "price": 20000, "price_payload": 20000, "price_fmt": "Rp20.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4"], "option_names": ["maung wisuda"], "option_names_raw": ["maung wisuda"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/17559de5f5f846daa12442c61d6f21c9~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/17559de5f5f846daa12442c61d6f21c9~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103342790919", "product_name": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - galih", "product_name_raw": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - galih", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441199370", "price": 20000, "price_payload": 20000, "price_fmt": "Rp20.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["5"], "option_names": ["galih"], "option_names_raw": ["galih"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/1e5c62974cfe4f06848cd22418272c87~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/1e5c62974cfe4f06848cd22418272c87~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103342790920", "product_name": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - merak", "product_name_raw": "3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY - merak", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441264906", "price": 20000, "price_payload": 20000, "price_fmt": "Rp20.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["6"], "option_names": ["merak"], "option_names_raw": ["merak"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/3de569aff3154f90840bf0a9ecfb4ff9~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/3de569aff3154f90840bf0a9ecfb4ff9~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
         </is>
       </c>
-      <c r="AP7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AS7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT7" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr">
+      <c r="AU7" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:19:09+07:00</t>
-        </is>
-      </c>
-      <c r="AT7" t="inlineStr">
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:42+07:00</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1951,58 +2124,88 @@
 Finishing menggunakan hand painting</t>
         </is>
       </c>
-      <c r="AI8" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=t%2BLknu0CWcUWk13YnZIIHDJOl6U%3D&amp;x-signature-webp=XDg%2B6AwCrmhFMLEce4DQOs3Inmk%3D</t>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material : PLA
+Size: 12cm
+Layer height : 0.2mm
+WAKTU PRODUKSI :
+Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.
+NOTE :
+- Pastikan file dapat di buka dan tidak error (png, JPEG, STP)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket.
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.
+TERMS &amp; CONDITION :
+- Pose atau gaya bisa disesuaikan dengan foto referensi
+- Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi.
+Finishing menggunakan hand painting</t>
         </is>
       </c>
       <c r="AJ8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material : PLA\nSize: 12cm\nLayer height : 0.2mm", "lines": ["Material : PLA", "Size: 12cm", "Layer height : 0.2mm"], "bullets": []}, {"section_no": 3, "title": "WAKTU PRODUKSI", "text": "Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.", "lines": ["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi."], "bullets": []}, {"section_no": 4, "title": "NOTE", "text": "- Pastikan file dapat di buka dan tidak error (png, JPEG, STP)\n- Maksimal revisi adalah sebelum masuk masa cetak\n- Warna dilakukan secara manual menggunakan cat akrilik\n- Ketika menerima paket, mohon rekam proses saat membuka paket.\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.", "lines": ["- Pastikan file dapat di buka dan tidak error (png, JPEG, STP)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket.", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."], "bullets": ["Pastikan file dapat di buka dan tidak error (png, JPEG, STP)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket."]}, {"section_no": 5, "title": "TERMS &amp; CONDITION", "text": "- Pose atau gaya bisa disesuaikan dengan foto referensi\n- Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi.\nFinishing menggunakan hand painting", "lines": ["- Pose atau gaya bisa disesuaikan dengan foto referensi", "- Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi.", "Finishing menggunakan hand painting"], "bullets": ["Pose atau gaya bisa disesuaikan dengan foto referensi", "Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi."]}]</t>
+        </is>
+      </c>
+      <c r="AL8" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Efci3BJtcP1Nh8%2F41pcOhqiXuIE%3D&amp;x-signature-webp=YMLls2p9Rh%2B8LkdlWOHSZPfXazk%3D</t>
+        </is>
+      </c>
+      <c r="AM8" t="n">
         <v>3</v>
       </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=t%2BLknu0CWcUWk13YnZIIHDJOl6U%3D&amp;x-signature-webp=XDg%2B6AwCrmhFMLEce4DQOs3Inmk%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=PE9y%2BTMK3jdlhFzrfu2YpWI1I%2FQ%3D&amp;x-signature-webp=rXQG8RhZQfjCwwNbJ6yXGeD%2Fsj4%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=7xj5hESN8V2BmNlbxzQRgxWcICQ%3D&amp;x-signature-webp=MtcaHaC%2FZ0yNQJ1r2EpctEn1Qko%3D"]</t>
-        </is>
-      </c>
-      <c r="AL8" t="inlineStr">
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Efci3BJtcP1Nh8%2F41pcOhqiXuIE%3D&amp;x-signature-webp=YMLls2p9Rh%2B8LkdlWOHSZPfXazk%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Dkf9Gkw4AxdKLRM0Xj4U%2FDJ9HOY%3D&amp;x-signature-webp=PeyEebN5r1EI9Ivoz14wZs3F1v0%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Xd2mVZHSwsaoWFzptDfGC3JldGQ%3D&amp;x-signature-webp=zKd5ebneXXRuS9qC1lztMv9kpzU%3D"]</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
         <is>
           <t>Niuva_Product_Images\103340568955\gallery_001.jpg</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AP8" t="inlineStr">
         <is>
           <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Figure Set"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
         </is>
       </c>
-      <c r="AN8" t="inlineStr">
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>[{"name": "finishing", "identifier": "", "options": [{"option_id": "2", "value": "NO COLOUR", "hex_color": "", "stock": 5, "picture_url": "", "picture_url_100": ""}, {"option_id": "3", "value": "COLOUR (Acrylic hand painting)", "hex_color": "", "stock": 5, "picture_url": "", "picture_url_100": ""}]}]</t>
         </is>
       </c>
-      <c r="AO8" t="inlineStr">
+      <c r="AR8" t="inlineStr">
         <is>
           <t>[{"product_id": "103340568955", "product_name": "3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll) - NO COLOUR", "product_name_raw": "3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll) - NO COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762", "price": 35200, "price_payload": 35200, "price_fmt": "Rp35.200", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["2"], "option_names": ["NO COLOUR"], "option_names_raw": ["NO COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f2998fb257e94aa18a47108f1861705e~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f2998fb257e94aa18a47108f1861705e~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103340568956", "product_name": "3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll) - COLOUR (Acrylic hand painting)", "product_name_raw": "3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll) - COLOUR (Acrylic hand painting)", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722988298", "price": 124800, "price_payload": 124800, "price_fmt": "Rp124.800", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3"], "option_names": ["COLOUR (Acrylic hand painting)"], "option_names_raw": ["COLOUR (Acrylic hand painting)"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f2998fb257e94aa18a47108f1861705e~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f2998fb257e94aa18a47108f1861705e~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
         </is>
       </c>
-      <c r="AP8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AS8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT8" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr">
+      <c r="AU8" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:19:20+07:00</t>
-        </is>
-      </c>
-      <c r="AT8" t="inlineStr">
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:45+07:00</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2137,15 +2340,36 @@
 - Warna dilakukan secara manual menggunakan cat akrilik
 - Ketika menerima paket, mohon rekam proses saat membuka paket.
 PRE ORDER CUSTOM ORDER
-Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan 
-Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu 
+Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan
+Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu
 Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
 Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
         </is>
       </c>
-      <c r="AI9" s="2" t="inlineStr">
-        <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=WI%2BmGBMcNKHVwFjKOlIuXlvfYCs%3D&amp;x-signature-webp=WdUTi75634FjssOYBX5fYA13RgQ%3D</t>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!
+DETAIL PRODUK :
+Material : PLA
+Size: 12cm
+Layer height : 0.2mm
+WAKTU PRODUKSI :
+Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.
+TERMS &amp; CONDITION :
+- Pose atau gaya bisa disesuaikan dengan foto referensi
+- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.
+- Finishing menggunakan hand painting
+NOTE :
+- Pastikan file dapat di buka dan tidak error (png, JPEG, STL)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket.
+PRE ORDER CUSTOM ORDER
+Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan
+Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu
+Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
         </is>
       </c>
       <c r="AJ9" t="n">
@@ -2153,72 +2377,85 @@
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=WI%2BmGBMcNKHVwFjKOlIuXlvfYCs%3D&amp;x-signature-webp=WdUTi75634FjssOYBX5fYA13RgQ%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=8p3LU9ULew1tA6kHyThPuUY%2BCK0%3D&amp;x-signature-webp=VnZqmwhR8zB5P2OrF0HPj1c83uo%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=7D4Zbq9RA7TAxtuczetEF04Nyj0%3D&amp;x-signature-webp=nmeBl5FzXCci8wbiEqZKvSENJfI%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=AiQYogKrI3ZKM7OCLoF7mF%2BXt3M%3D&amp;x-signature-webp=%2BH9Si15hpZah3hrDCUrMfB1igdg%3D", "https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=ZU0AiqbegW%2BpfBRTg3wvrmQ3a5M%3D&amp;x-signature-webp=dara6IKBD2z7%2BEwfHNKwsHdqtOc%3D"]</t>
-        </is>
-      </c>
-      <c r="AL9" t="inlineStr">
+          <t>[{"section_no": 1, "title": "DESKRIPSI UMUM", "text": "NIUVA STUDIO – Jasa 3D print custom\nNiuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!", "lines": ["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"], "bullets": []}, {"section_no": 2, "title": "DETAIL PRODUK", "text": "Material : PLA\nSize: 12cm\nLayer height : 0.2mm", "lines": ["Material : PLA", "Size: 12cm", "Layer height : 0.2mm"], "bullets": []}, {"section_no": 3, "title": "WAKTU PRODUKSI", "text": "Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.", "lines": ["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi."], "bullets": []}, {"section_no": 4, "title": "TERMS &amp; CONDITION", "text": "- Pose atau gaya bisa disesuaikan dengan foto referensi\n- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.\n- Finishing menggunakan hand painting", "lines": ["- Pose atau gaya bisa disesuaikan dengan foto referensi", "- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.", "- Finishing menggunakan hand painting"], "bullets": ["Pose atau gaya bisa disesuaikan dengan foto referensi", "Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.", "Finishing menggunakan hand painting"]}, {"section_no": 5, "title": "NOTE", "text": "- Pastikan file dapat di buka dan tidak error (png, JPEG, STL)\n- Maksimal revisi adalah sebelum masuk masa cetak\n- Warna dilakukan secara manual menggunakan cat akrilik\n- Ketika menerima paket, mohon rekam proses saat membuka paket.\nPRE ORDER CUSTOM ORDER\nProduksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan\nUntuk Pre-Order, customer WAJIB chat admin terlebih dahulu\nPembayaran full 3 hari sebelum delivery (tidak ada deposit)\nJika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.", "lines": ["- Pastikan file dapat di buka dan tidak error (png, JPEG, STL)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket.", "PRE ORDER CUSTOM ORDER", "Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan", "Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu", "Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."], "bullets": ["Pastikan file dapat di buka dan tidak error (png, JPEG, STL)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket."]}]</t>
+        </is>
+      </c>
+      <c r="AL9" s="2" t="inlineStr">
+        <is>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=JzuGZkBT%2FivUuAES754e3G7xEBg%3D&amp;x-signature-webp=qU1UVGZCXDI2%2FoUWU2Wr2VrWYtg%3D</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>["https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=JzuGZkBT%2FivUuAES754e3G7xEBg%3D&amp;x-signature-webp=qU1UVGZCXDI2%2FoUWU2Wr2VrWYtg%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=0oAWPPB9%2FWirKROikDeV7UqZ%2BjY%3D&amp;x-signature-webp=J%2FTOGC%2BcIaDazz1DbxQKh8HTZGo%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=96AAJ2Sx9khmvt2Pc2vksX4Nbjk%3D&amp;x-signature-webp=Pbx0bxSLhIfoYM2cPbQH%2Fkaeg5c%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=6HKct0z0vV8o6rt0dlS97YnX4rM%3D&amp;x-signature-webp=J%2B10JMv9SYpOR5szhoCfH8wd3Tk%3D", "https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=zxq4qogcgI2kpsBJOUDVUmnBhVc%3D&amp;x-signature-webp=JQRRUOHHKFymUqK%2F1ajq7QEDUiM%3D"]</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
         <is>
           <t>Niuva_Product_Images\103339597166\gallery_001.jpg</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr">
+      <c r="AP9" t="inlineStr">
         <is>
           <t>[{"title": "Kondisi", "value": "Baru"}, {"title": "Pemesanan Minimum", "value": "1 Buah"}, {"title": "Kategori", "value": "Figure Set"}, {"title": "Etalase", "value": "Semua Etalase"}]</t>
         </is>
       </c>
-      <c r="AN9" t="inlineStr">
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>[{"name": "style", "identifier": "", "options": [{"option_id": "3", "value": "CARTOON", "hex_color": "", "stock": 10, "picture_url": "", "picture_url_100": ""}, {"option_id": "4", "value": "EMOJI", "hex_color": "", "stock": 10, "picture_url": "", "picture_url_100": ""}, {"option_id": "5", "value": "PETITE", "hex_color": "", "stock": 10, "picture_url": "", "picture_url_100": ""}, {"option_id": "6", "value": "BIG HEAD", "hex_color": "", "stock": 10, "picture_url": "", "picture_url_100": ""}]}, {"name": "finishing", "identifier": "", "options": [{"option_id": "7", "value": "NO COLOUR", "hex_color": "", "stock": 0, "picture_url": "", "picture_url_100": ""}, {"option_id": "8", "value": "COLOUR", "hex_color": "", "stock": 0, "picture_url": "", "picture_url_100": ""}]}]</t>
         </is>
       </c>
-      <c r="AO9" t="inlineStr">
+      <c r="AR9" t="inlineStr">
         <is>
           <t>[{"product_id": "103339597166", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - CARTOON, NO COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - CARTOON, NO COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858", "price": 35200, "price_payload": 35200, "price_fmt": "Rp35.200", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3", "7"], "option_names": ["CARTOON", "NO COLOUR"], "option_names_raw": ["CARTOON", "NO COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597167", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - CARTOON, COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - CARTOON, COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156592394", "price": 124800, "price_payload": 124800, "price_fmt": "Rp124.800", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["3", "8"], "option_names": ["CARTOON", "COLOUR"], "option_names_raw": ["CARTOON", "COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597168", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - EMOJI, NO COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - EMOJI, NO COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156657930", "price": 70000, "price_payload": 70000, "price_fmt": "Rp70.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4", "7"], "option_names": ["EMOJI", "NO COLOUR"], "option_names_raw": ["EMOJI", "NO COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597169", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - EMOJI, COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - EMOJI, COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156723466", "price": 160000, "price_payload": 160000, "price_fmt": "Rp160.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["4", "8"], "option_names": ["EMOJI", "COLOUR"], "option_names_raw": ["EMOJI", "COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597170", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - PETITE, NO COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - PETITE, NO COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156789002", "price": 70000, "price_payload": 70000, "price_fmt": "Rp70.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["5", "7"], "option_names": ["PETITE", "NO COLOUR"], "option_names_raw": ["PETITE", "NO COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597171", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - PETITE, COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - PETITE, COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156854538", "price": 160000, "price_payload": 160000, "price_fmt": "Rp160.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["5", "8"], "option_names": ["PETITE", "COLOUR"], "option_names_raw": ["PETITE", "COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597172", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - BIG HEAD, NO COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - BIG HEAD, NO COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156920074", "price": 42000, "price_payload": 42000, "price_fmt": "Rp42.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["6", "7"], "option_names": ["BIG HEAD", "NO COLOUR"], "option_names_raw": ["BIG HEAD", "NO COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}, {"product_id": "103339597173", "product_name": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - BIG HEAD, COLOUR", "product_name_raw": "[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER - BIG HEAD, COLOUR", "product_url": "https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156985610", "price": 132000, "price_payload": 132000, "price_fmt": "Rp132.000", "original_price": null, "slash_price_fmt": "", "discount_percentage": 0.0, "option_ids": ["6", "8"], "option_names": ["BIG HEAD", "COLOUR"], "option_names_raw": ["BIG HEAD", "COLOUR"], "stock": 5, "is_buyable": true, "minimum_order": 1, "maximum_order": 5, "stock_message": "Stok tersisa beli segera!", "is_cod": false, "image_url": "https://images.tokopedia.net/img/cache/700/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg.webp", "image_url_100": "https://images.tokopedia.net/img/cache/150/aphluv/1997/1/1/f459dd5b748e424e9c656220f3bc9b12~.jpeg", "is_placeholder": false, "status": "TERSEDIA"}]</t>
         </is>
       </c>
-      <c r="AP9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ9" t="inlineStr">
+      <c r="AS9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT9" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
+      <c r="AU9" t="inlineStr">
         <is>
           <t>apollo_cache</t>
         </is>
       </c>
-      <c r="AS9" t="inlineStr">
-        <is>
-          <t>2026-09-17T04:19:23+07:00</t>
-        </is>
-      </c>
-      <c r="AT9" t="inlineStr">
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:53:47+07:00</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AU9"/>
+  <autoFilter ref="A1:AX9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AI9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2494,7 +2731,7 @@
       <c r="J2" s="3" t="n">
         <v>95000</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L2" t="inlineStr">
@@ -2627,7 +2864,7 @@
       <c r="J3" s="3" t="n">
         <v>75000</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="3" t="n">
         <v>75000</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -2760,7 +2997,7 @@
       <c r="J4" s="3" t="n">
         <v>85000</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="3" t="n">
         <v>85000</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -2893,7 +3130,7 @@
       <c r="J5" s="3" t="n">
         <v>65000</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="3" t="n">
         <v>65000</v>
       </c>
       <c r="L5" t="inlineStr">
@@ -3026,7 +3263,7 @@
       <c r="J6" s="3" t="n">
         <v>65000</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="3" t="n">
         <v>65000</v>
       </c>
       <c r="L6" t="inlineStr">
@@ -3159,7 +3396,7 @@
       <c r="J7" s="3" t="n">
         <v>45000</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="3" t="n">
         <v>45000</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -3292,7 +3529,7 @@
       <c r="J8" s="3" t="n">
         <v>80000</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="3" t="n">
         <v>80000</v>
       </c>
       <c r="L8" t="inlineStr">
@@ -3425,7 +3662,7 @@
       <c r="J9" s="3" t="n">
         <v>60000</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -3558,7 +3795,7 @@
       <c r="J10" s="3" t="n">
         <v>150000</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="3" t="n">
         <v>150000</v>
       </c>
       <c r="L10" t="inlineStr">
@@ -3691,7 +3928,7 @@
       <c r="J11" s="3" t="n">
         <v>80000</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="3" t="n">
         <v>80000</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -3824,7 +4061,7 @@
       <c r="J12" s="3" t="n">
         <v>55000</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="3" t="n">
         <v>55000</v>
       </c>
       <c r="L12" t="inlineStr">
@@ -3957,7 +4194,7 @@
       <c r="J13" s="3" t="n">
         <v>35000</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="3" t="n">
         <v>35000</v>
       </c>
       <c r="L13" t="inlineStr">
@@ -4083,7 +4320,7 @@
         </is>
       </c>
       <c r="J14" s="3" t="n"/>
-      <c r="K14" t="n">
+      <c r="K14" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -4202,7 +4439,7 @@
         </is>
       </c>
       <c r="J15" s="3" t="n"/>
-      <c r="K15" t="n">
+      <c r="K15" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -4321,7 +4558,7 @@
         </is>
       </c>
       <c r="J16" s="3" t="n"/>
-      <c r="K16" t="n">
+      <c r="K16" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -4440,7 +4677,7 @@
         </is>
       </c>
       <c r="J17" s="3" t="n"/>
-      <c r="K17" t="n">
+      <c r="K17" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -4559,7 +4796,7 @@
         </is>
       </c>
       <c r="J18" s="3" t="n"/>
-      <c r="K18" t="n">
+      <c r="K18" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -4678,7 +4915,7 @@
         </is>
       </c>
       <c r="J19" s="3" t="n"/>
-      <c r="K19" t="n">
+      <c r="K19" s="3" t="n">
         <v>95000</v>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -4804,7 +5041,7 @@
       <c r="J20" s="3" t="n">
         <v>35200</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="3" t="n">
         <v>35200</v>
       </c>
       <c r="L20" t="inlineStr">
@@ -4927,7 +5164,7 @@
       <c r="J21" s="3" t="n">
         <v>30400</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="3" t="n">
         <v>30400</v>
       </c>
       <c r="L21" t="inlineStr">
@@ -5050,7 +5287,7 @@
       <c r="J22" s="3" t="n">
         <v>30400</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="3" t="n">
         <v>30400</v>
       </c>
       <c r="L22" t="inlineStr">
@@ -5173,7 +5410,7 @@
       <c r="J23" s="3" t="n">
         <v>150000</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" s="3" t="n">
         <v>150000</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -5296,7 +5533,7 @@
       <c r="J24" s="3" t="n">
         <v>150000</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" s="3" t="n">
         <v>150000</v>
       </c>
       <c r="L24" t="inlineStr">
@@ -5419,7 +5656,7 @@
       <c r="J25" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="L25" t="inlineStr">
@@ -5542,7 +5779,7 @@
       <c r="J26" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K26" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="L26" t="inlineStr">
@@ -5665,7 +5902,7 @@
       <c r="J27" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="L27" t="inlineStr">
@@ -5788,7 +6025,7 @@
       <c r="J28" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -5911,7 +6148,7 @@
       <c r="J29" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="L29" t="inlineStr">
@@ -6034,7 +6271,7 @@
       <c r="J30" s="3" t="n">
         <v>35200</v>
       </c>
-      <c r="K30" t="n">
+      <c r="K30" s="3" t="n">
         <v>35200</v>
       </c>
       <c r="L30" t="inlineStr">
@@ -6157,7 +6394,7 @@
       <c r="J31" s="3" t="n">
         <v>124800</v>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" s="3" t="n">
         <v>124800</v>
       </c>
       <c r="L31" t="inlineStr">
@@ -6280,7 +6517,7 @@
       <c r="J32" s="3" t="n">
         <v>35200</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K32" s="3" t="n">
         <v>35200</v>
       </c>
       <c r="L32" t="inlineStr">
@@ -6413,7 +6650,7 @@
       <c r="J33" s="3" t="n">
         <v>124800</v>
       </c>
-      <c r="K33" t="n">
+      <c r="K33" s="3" t="n">
         <v>124800</v>
       </c>
       <c r="L33" t="inlineStr">
@@ -6546,7 +6783,7 @@
       <c r="J34" s="3" t="n">
         <v>70000</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K34" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="L34" t="inlineStr">
@@ -6679,7 +6916,7 @@
       <c r="J35" s="3" t="n">
         <v>160000</v>
       </c>
-      <c r="K35" t="n">
+      <c r="K35" s="3" t="n">
         <v>160000</v>
       </c>
       <c r="L35" t="inlineStr">
@@ -6812,7 +7049,7 @@
       <c r="J36" s="3" t="n">
         <v>70000</v>
       </c>
-      <c r="K36" t="n">
+      <c r="K36" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="L36" t="inlineStr">
@@ -6945,7 +7182,7 @@
       <c r="J37" s="3" t="n">
         <v>160000</v>
       </c>
-      <c r="K37" t="n">
+      <c r="K37" s="3" t="n">
         <v>160000</v>
       </c>
       <c r="L37" t="inlineStr">
@@ -7078,7 +7315,7 @@
       <c r="J38" s="3" t="n">
         <v>42000</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K38" s="3" t="n">
         <v>42000</v>
       </c>
       <c r="L38" t="inlineStr">
@@ -7211,7 +7448,7 @@
       <c r="J39" s="3" t="n">
         <v>132000</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K39" s="3" t="n">
         <v>132000</v>
       </c>
       <c r="L39" t="inlineStr">
@@ -7457,6 +7694,1574 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>parent_product_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>parent_nama_produk</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>parent_url_produk</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>detail_no</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bagian_detail</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>detail_text</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>detail_lines_json</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>detail_bullets_json</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sumber_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>103726663896</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kicau Mania Kunci Gantung Kucing Lucu dengan Desain Kreatif dan Warna Cerah untuk Penggemar Kucing dan Aksesori Unik</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/kicau-mania-kunci-gantung-kucing-lucu-dengan-desain-kreatif-dan-warna-cerah-untuk-penggemar-kucing-dan-aksesori-unik-1737002078292313866</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk Merchandise lucu berbasis 3D print!</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk Merchandise lucu berbasis 3D print!"]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>103726663896</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kicau Mania Kunci Gantung Kucing Lucu dengan Desain Kreatif dan Warna Cerah untuk Penggemar Kucing dan Aksesori Unik</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/kicau-mania-kunci-gantung-kucing-lucu-dengan-desain-kreatif-dan-warna-cerah-untuk-penggemar-kucing-dan-aksesori-unik-1737002078292313866</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Material: PLA, Multicolor Print
+Size: 8 cm</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["Material: PLA, Multicolor Print", "Size: 8 cm"]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>103726663896</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kicau Mania Kunci Gantung Kucing Lucu dengan Desain Kreatif dan Warna Cerah untuk Penggemar Kucing dan Aksesori Unik</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/kicau-mania-kunci-gantung-kucing-lucu-dengan-desain-kreatif-dan-warna-cerah-untuk-penggemar-kucing-dan-aksesori-unik-1737002078292313866</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WAKTU PRODUKSI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.
+~2–3 hari</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.", "~2–3 hari"]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>103726663896</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kicau Mania Kunci Gantung Kucing Lucu dengan Desain Kreatif dan Warna Cerah untuk Penggemar Kucing dan Aksesori Unik</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/kicau-mania-kunci-gantung-kucing-lucu-dengan-desain-kreatif-dan-warna-cerah-untuk-penggemar-kucing-dan-aksesori-unik-1737002078292313866</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TERMS &amp; CONDITION</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>- Refund tidak akan diterima apabila tidak ada video unboxing</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["- Refund tidak akan diterima apabila tidak ada video unboxing"]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>["Refund tidak akan diterima apabila tidak ada video unboxing"]</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>103726663896</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kicau Mania Kunci Gantung Kucing Lucu dengan Desain Kreatif dan Warna Cerah untuk Penggemar Kucing dan Aksesori Unik</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/kicau-mania-kunci-gantung-kucing-lucu-dengan-desain-kreatif-dan-warna-cerah-untuk-penggemar-kucing-dan-aksesori-unik-1737002078292313866</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>- Ketika menerima paket, mohon rekam proses saat membuka paket</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["- Ketika menerima paket, mohon rekam proses saat membuka paket"]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>["Ketika menerima paket, mohon rekam proses saat membuka paket"]</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Variasi Figur Full-Color (Paint)
+Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 15 cm, 12 cm
+Variasi Figur Single Color
+Material: PLA, Single Color Print
+Size: 15 cm, 12 cm
+Variasi Lego Full-Color (Paint)
+Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 12 cm, 8 cm
+Variasi Lego Full-Color (MultiColor Print)
+Material: PLA, Multi-Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish
+Size: 12 cm, 8 cm
+Variasi Lego Single Color
+Material: PLA, Single Color Print
+Size: 12 cm, 8 cm</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["Variasi Figur Full-Color (Paint)", "Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 15 cm, 12 cm", "Variasi Figur Single Color", "Material: PLA, Single Color Print", "Size: 15 cm, 12 cm", "Variasi Lego Full-Color (Paint)", "Material: PLA, Single Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 12 cm, 8 cm", "Variasi Lego Full-Color (MultiColor Print)", "Material: PLA, Multi-Color Print, Hand-Painted with Acrylic Paint and Clear Spray Paint (Matte/Glossy) Finish", "Size: 12 cm, 8 cm", "Variasi Lego Single Color", "Material: PLA, Single Color Print", "Size: 12 cm, 8 cm"]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WAKTU PRODUKSI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Estimasi penyelesaian mengikuti durasi printing, custom paint job, dan kondisi antrian produksi.
+~6–7 hari</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["Estimasi penyelesaian mengikuti durasi printing, custom paint job, dan kondisi antrian produksi.", "~6–7 hari"]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TERMS &amp; CONDITION</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi
+- Finishing menggunakan hand painting
+- Refund tidak akan diterima apabila tidak ada video unboxing</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi", "- Finishing menggunakan hand painting", "- Refund tidak akan diterima apabila tidak ada video unboxing"]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>["Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi", "Finishing menggunakan hand painting", "Refund tidak akan diterima apabila tidak ada video unboxing"]</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>- Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["- Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket"]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>["Pastikan foto referensi dapat di buka dan tidak error (PNG, JPEG)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket"]</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>103726333343</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wisuda Custom 3D Print - Patung Graduasi 3D Personalisasi untuk Souvenir Khusus</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/wisuda-custom-3d-print-patung-graduasi-3d-personalisasi-untuk-souvenir-khusus-1737001056781305610-1737001528663770890</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PRE ORDER CUSTOM ORDER</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan
+- Untuk pesanan custom customer WAJIB chat admin terlebih dahulu
+- Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
+- Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>["- Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan", "- Untuk pesanan custom customer WAJIB chat admin terlebih dahulu", "- Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "- Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>["Produksi akan memakan waktu 6–7 hari, tergantung besar/kecil produk dan lama pengecatan", "Untuk pesanan custom customer WAJIB chat admin terlebih dahulu", "Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."]</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>103474501379</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3D PRINT LEGO FIGURE WISUDAWAN TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-1736031180211586826</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO - Jasa 3D print custom
+Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO - Jasa 3D print custom", "Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>103474501379</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3D PRINT LEGO FIGURE WISUDAWAN TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-1736031180211586826</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Material: PLA
+Size: 12cm
+Layer height : 0.2mm</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>["Material: PLA", "Size: 12cm", "Layer height : 0.2mm"]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>103474501379</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>3D PRINT LEGO FIGURE WISUDAWAN TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-1736031180211586826</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>- tulis fakultas di notes/chat yaa
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.
+Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>["- tulis fakultas di notes/chat yaa", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.", "Komplain tanpa bukti video tidak dapat diproses"]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>["tulis fakultas di notes/chat yaa"]</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>103343689816</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>103343689816</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN GEDUNG TELKOM UNIVERSITY (TULT, BANDUNG TECHNO PARK)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-gedung-telkom-university-tult-bandung-techno-park-1735431958738929418-1735431963114374922</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Material : PLA
+Size: 8cm
+Layer height : 0.2mm
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>["Material : PLA", "Size: 8cm", "Layer height : 0.2mm", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses"]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>103343687481</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO - Jasa 3D print custom
+Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO - Jasa 3D print custom", "Niuva Inovasi Utama - Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>103343687481</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Material: PLA
+Size: 12cm
+Layer height : 0.2mm</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>["Material: PLA", "Size: 12cm", "Layer height : 0.2mm"]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>103343687481</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3D Print LEGO Figure Wisudawan Telkom University PLA (Bisa Custom Tali Toga Fakultas)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-lego-figure-wisudawan-telkom-university-pla-bisa-custom-tali-toga-fakultas-1735433388996069130-1735433427198904074</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>- tulis fakultas di notes/chat yaa
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.
+Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>["- tulis fakultas di notes/chat yaa", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti.", "Komplain tanpa bukti video tidak dapat diproses"]</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>["tulis fakultas di notes/chat yaa"]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>103342790916</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441002762</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>103342790916</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3D PRINT KEYCHAIN ANIMAL TELKOM UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-keychain-animal-telkom-university-1735431904246466314-1735431958441002762</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Material : PLA
+Size: 8cm
+Layer height : 0.2mm
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>["Material : PLA", "Size: 8cm", "Layer height : 0.2mm", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses"]</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>103340568955</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>103340568955</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Material : PLA
+Size: 12cm
+Layer height : 0.2mm</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>["Material : PLA", "Size: 12cm", "Layer height : 0.2mm"]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>103340568955</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>WAKTU PRODUKSI</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi."]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>103340568955</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>- Pastikan file dapat di buka dan tidak error (png, JPEG, STP)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket.
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>["- Pastikan file dapat di buka dan tidak error (png, JPEG, STP)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket.", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>["Pastikan file dapat di buka dan tidak error (png, JPEG, STP)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket."]</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>103340568955</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>3D PRINT CUSTOM FIGURE SPECIAL MOMENTS (Newborn, weddings, birthday, dll)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-special-moments-newborn-weddings-birthday-dll-1735422370974500618-1735423689722922762</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TERMS &amp; CONDITION</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>- Pose atau gaya bisa disesuaikan dengan foto referensi
+- Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi.
+Finishing menggunakan hand painting</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>["- Pose atau gaya bisa disesuaikan dengan foto referensi", "- Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi.", "Finishing menggunakan hand painting"]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>["Pose atau gaya bisa disesuaikan dengan foto referensi", "Desain yang sudah fix dan sudah memasuki - - tahap cetak tidak bisa revisi lagi."]</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>103339597166</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>DESKRIPSI UMUM</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NIUVA STUDIO – Jasa 3D print custom
+Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>["NIUVA STUDIO – Jasa 3D print custom", "Niuva Inovasi Utama – Niuva Studio merupakan mitra strategis inovasi dan pengembangan produk. Kami menghadirkan solusi kreatif berbasis riset dari konsultasi untuk menciptakan nilai tambah dan keunggulan yang nyata. Salah satu bentuknya adalah produk berbasis 3D print yang kami tawarkan untuk mengabadikan Special Moments mu!"]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>103339597166</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>DETAIL PRODUK</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Material : PLA
+Size: 12cm
+Layer height : 0.2mm</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>["Material : PLA", "Size: 12cm", "Layer height : 0.2mm"]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>103339597166</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>WAKTU PRODUKSI</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>["Estimasi penyelesaian mengikuti durasi printing dan kondisi antrian produksi."]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>103339597166</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TERMS &amp; CONDITION</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>- Pose atau gaya bisa disesuaikan dengan foto referensi
+- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.
+- Finishing menggunakan hand painting</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>["- Pose atau gaya bisa disesuaikan dengan foto referensi", "- Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.", "- Finishing menggunakan hand painting"]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>["Pose atau gaya bisa disesuaikan dengan foto referensi", "Desain yang sudah fix dan sudah memasuki tahap cetak tidak bisa revisi lagi.", "Finishing menggunakan hand painting"]</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>103339597166</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>[PREORDER] 3D PRINT CUSTOM FIGURE (Bubble head, chibi, cartoon, emoji) READ DESCRIPTION FOR ORDER</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tokopedia.com/niuvastudio/3d-print-custom-figure-bubble-head-chibi-cartoon-emoji-1735421281506264842-1735421539156526858</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>- Pastikan file dapat di buka dan tidak error (png, JPEG, STL)
+- Maksimal revisi adalah sebelum masuk masa cetak
+- Warna dilakukan secara manual menggunakan cat akrilik
+- Ketika menerima paket, mohon rekam proses saat membuka paket.
+PRE ORDER CUSTOM ORDER
+Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan
+Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu
+Pembayaran full 3 hari sebelum delivery (tidak ada deposit)
+Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>["- Pastikan file dapat di buka dan tidak error (png, JPEG, STL)", "- Maksimal revisi adalah sebelum masuk masa cetak", "- Warna dilakukan secara manual menggunakan cat akrilik", "- Ketika menerima paket, mohon rekam proses saat membuka paket.", "PRE ORDER CUSTOM ORDER", "Produksi akan memakan waktu 1-2 minggu, tergantung besar/kecil produk dan lama pengecatan", "Untuk Pre-Order, customer WAJIB chat admin terlebih dahulu", "Pembayaran full 3 hari sebelum delivery (tidak ada deposit)", "Jika ada kesalahan pengiriman atau kekurangan barang, silakan hubungi kami dan sertakan video sebagai bukti. Komplain tanpa bukti video tidak dapat diproses."]</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>["Pastikan file dapat di buka dan tidak error (png, JPEG, STL)", "Maksimal revisi adalah sebelum masuk masa cetak", "Warna dilakukan secara manual menggunakan cat akrilik", "Ketika menerima paket, mohon rekam proses saat membuka paket."]</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>apollo_cache</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I32"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7579,12 +9384,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=svD%2FMCbTAPMm2sw3axtTVj4uNsk%3D&amp;x-signature-webp=UiNX8Pb8pX4wBN4ZqxAXqh%2BYC4c%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=4UISL%2FYJboBGuHt6v1SbO9Ryzwk%3D&amp;x-signature-webp=Jo2zBlT%2BgGlMuyjqqgYIkNt3UyA%3D</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=J6Av%2BTl%2FWtC5hC7w%2BcTiMLOX4no%3D&amp;x-signature-webp=x%2FavwygptYz4E5r7O1cO1bkhIRk%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/73ea006d34cf4944bcbf7040035b2ab1~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=m7a7cv1obktU0FMXzYM2RWcgNHM%3D&amp;x-signature-webp=EQS%2FTjEAn7bhjvsC5N3%2B7X7%2FO2U%3D</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -7629,12 +9434,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=MkefKNp5%2B1oQyUlL6iDIw%2FA%2FDGo%3D&amp;x-signature-webp=OVc29sBMOGQ%2FvVZ6zaQfDfonGkw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=XsGpxpSDGKqY5l2EYJZ7b2Qgeik%3D&amp;x-signature-webp=usEfoIBSW4MdqQdPseXbIMLLmow%3D</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604334&amp;x-signature=qtKxboNZxo6Za3p%2B50eF3y%2FFhCw%3D&amp;x-signature-webp=A3SCgrRJIKA60jKI1zizvGwG7mo%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/eb84e3e85b4f43c5b279ae90d270f4c0~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646002&amp;x-signature=bqi%2Fu2XSI5cHBN7OfuyuCxaY9cU%3D&amp;x-signature-webp=Wj9E%2Ba62bUoPSzNI7YCuseVhR%2F4%3D</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -7679,12 +9484,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=2WvRYF4O2pDZ9vH2v9pFsbkwT48%3D&amp;x-signature-webp=oSOAwZPGCrxm8Nu4vSNrOJ5eAVA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=lVd4XUDpWS9eRMEqkfo%2BqooJq74%3D&amp;x-signature-webp=pp2yEsiGGIIvLKueQb1pY214YQU%3D</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=pXMuSnHtssYKd2usyOktS7XPCEs%3D&amp;x-signature-webp=v8q6tiXGlLE5GBeDtYV%2FdTWSVmk%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/70f78c7827e64a44ae2300b7a55eb96f~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=kGIAaxLzaet%2BI6Vq8dHkx%2BKXUQI%3D&amp;x-signature-webp=jx2BPxqF9NMD0EArbf93wpgSR5s%3D</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -7729,12 +9534,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=WifDo1nzytofLdD5KU9pC0YX9XM%3D&amp;x-signature-webp=OyHmfon9RRjJgo6DUeLWei6u8KM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=KdpLa3GULJtv9AjRZatL6whc7ZI%3D&amp;x-signature-webp=URFFCPLSgZ8vTlDuGkIqMN7ETHE%3D</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=NO5HGeOg5eeBUc6ff3QCDVPF2mA%3D&amp;x-signature-webp=N9b4SKU3Sd2Vn8ePZuixkPrcLns%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/2895518b3f3e437a99eb47ebe8d12387~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=th0f24u8dpPlQtq9aub2fUaUCnI%3D&amp;x-signature-webp=3fDAWw5GV3zePzpvFYN0%2FZSLB0c%3D</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -7779,12 +9584,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=ExrUTK1UrT3PT1vCvxLDUQiSVpE%3D&amp;x-signature-webp=3dFzitryP31qFGQe1oMbcGzPNdA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=qMIMIQ%2Bo9Mgb3pJUpi5eIuskNms%3D&amp;x-signature-webp=6nXxcwwjugD6xF1kR0NQuopW1Ls%3D</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=52lfMxQSWI5IhXIgEYYF6%2BvoKGU%3D&amp;x-signature-webp=pmJhWRgixjOxgdqw0%2BBYCs1vb5g%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/98abfe8b86c04aa391091e8549c9bd7a~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=EKOblb00oe6%2Fr0rSHq11FLYHPJc%3D&amp;x-signature-webp=avG6MWUQQ02CUIhy%2B7NfYpavav8%3D</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -7829,12 +9634,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=3yfqcRPVECTQmgx6ChjVxk4UyL4%3D&amp;x-signature-webp=%2FDhE3JoMTuPEinrSTr%2BeR2ViDg4%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=TN%2BmsynoafUSezIdHeIhIui9cX4%3D&amp;x-signature-webp=FXNOEUSt7bnwZgoN%2B3Upw5j%2BeWM%3D</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=duF%2FLJ%2FLYDG96OWTdMi%2B5OESHR0%3D&amp;x-signature-webp=YMUSYS%2BjrfJO5QyiCF5KsUl9oGc%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/953f4730e0cd4002af1024c33147fa80~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=%2F0j3EOlXSjzsCoGAp8MvmNEPzuE%3D&amp;x-signature-webp=WRk9vf6StT2%2BcGF%2F32zacMKJpoc%3D</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -7879,12 +9684,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=9h08J1k%2By7jEMSAN0j4xvKF64qo%3D&amp;x-signature-webp=a%2FvWKMkIZ0htfkAGWv2ncSirE1g%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=pCHyfVTtO2d%2FYQejpL4P3G4QSe0%3D&amp;x-signature-webp=7gu5N1oS%2FBIoRszbJ%2B3OyeRzuD8%3D</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604336&amp;x-signature=qwfRADK8upnWsHBbqOhhA%2B0SL6g%3D&amp;x-signature-webp=xJoKpO74iznrtDllAtUwf60kfbs%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8ecde87b876e4e9aa40a5bff368747ae~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646008&amp;x-signature=UulMm5ru4LkqauBflZdHCM686gQ%3D&amp;x-signature-webp=%2B5vQRpKQ02y7jN5ilntNgT8igK4%3D</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -8589,12 +10394,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=tqAdXHjGXCOUSW3eaHZLt9qaAvU%3D&amp;x-signature-webp=5HsayE8Hv1J7LrIcmqUE1TWGhpA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=j3QM%2Bnlx1YUB2%2Bd3r%2FYdkcPq%2Bjk%3D&amp;x-signature-webp=BDhDKtuKqO62qEOXTE8om5%2BGnTE%3D</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=gZutHo%2FRmSGUslDeDXhtygFS3CU%3D&amp;x-signature-webp=0awUwzdZPAsP63acXL7F182gLj4%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/8b099fd1aa4e49e2998ae999803708fa~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=SkKXutubu2608ERy1Jagrq%2Fx2kY%3D&amp;x-signature-webp=BwxjWvJ41iJko7k7Q7jV5fCEXsg%3D</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -8639,12 +10444,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=R8SMoLrgf6%2BEa6d9u6DfW8M82PM%3D&amp;x-signature-webp=zfwyhXJ3RrxAI%2BsPAPogPjJCG1k%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=A%2BLggcWo1DNN4xASKtWrj6m1XZY%3D&amp;x-signature-webp=d%2F1P%2Fpi3DYifmMwjKTW7HYXJCz0%3D</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604339&amp;x-signature=kZC6H98nNkvFMktS95uVUMmms1I%3D&amp;x-signature-webp=r7PBGgL8JNRtMYpYJEMRQ1UOBVc%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f3ebd02f8d3044808010eebaada7b8a0~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646011&amp;x-signature=PMfp288cBmkv%2Fde6izLKo66140E%3D&amp;x-signature-webp=Z7UYKogYAu1WwcpdQFkNtC9LDHE%3D</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -8689,12 +10494,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=Hh%2Bu8u%2FUdoOjIoP%2Fd1fMcWARPfs%3D&amp;x-signature-webp=aL0aZwXndr8wLDsEIVpjPk5284E%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=bSSq4nt%2B1%2BQjDqLw2xZ%2FF4DE6Z8%3D&amp;x-signature-webp=8n8x3kU2zcCyaMWhj70OApnJKJM%3D</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=O9Dr%2FPDMBF9G1BdhBEqRlZWc9Ak%3D&amp;x-signature-webp=fL%2BBZNlAtc4w%2BDr2%2Bfuqxe1pnr0%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4d1042ce0a4841c4b1cddde7c56e4253~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=%2BAIZjLL564zzYdvzD3PFJDGfAjU%3D&amp;x-signature-webp=q1UdDCveorZgJPPgqFvQIcj%2Bos0%3D</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -8739,12 +10544,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=0Hklwo%2BwJ0mQNelPLvc950PeWXU%3D&amp;x-signature-webp=BPq9W2FGcgi2edMK%2BfUTAgnlzlw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=Enc4sPipEhn9qLy%2BX4Hw4ZNBOO4%3D&amp;x-signature-webp=%2FiyRGB8bTXq3JFHOKx7XGzQlv9s%3D</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=lzh0Viw92pdhjn72UaR5orSkT4Y%3D&amp;x-signature-webp=PvcmrQ%2F6fgELDnxekiHmOUgEQd4%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5197b144621c4b56bc569b2712dd84a7~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=yxR%2BU6Ek6G3rmYSAscjGj9jO5Ps%3D&amp;x-signature-webp=Zxg%2BE8HbxhEjnEg0SbPKoKOCLJg%3D</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -8789,12 +10594,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=8JLonBXZnCN8wAn3EjLeDlRilvw%3D&amp;x-signature-webp=PoDzEMvYgyuCCCzT2htgMymxQ4s%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=S0V9KaIXwAAUyiWNXU%2FzcTTewmg%3D&amp;x-signature-webp=%2BDyuTyDAvzVRTwIUnNFp5Sp2gAI%3D</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=2g8K6FKw3OuyqzgIkMECFgISh7g%3D&amp;x-signature-webp=oeB%2F4R%2F9GFH0DBS%2FXDWu6te2MV0%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d645dd79b9564e0ca37bde219012b21b~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=dFqlh4V1eOM9GuaXa65ur5UpYMc%3D&amp;x-signature-webp=Kp2hePvF17SN0PrzMIEBPP4v99M%3D</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -8839,12 +10644,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=Mk6p9D7Q7BJ%2B2hiNdPqoQz5w4i0%3D&amp;x-signature-webp=0QRT5j6ABMvHZG20oa6F24scQFU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=gjB3D6cjx7Uf7vIuqJNjUJz6Lao%3D&amp;x-signature-webp=olv1eG3Z6fgGkeHTVLVG9BJVsIg%3D</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=ndHdDPa5LUaKuq%2FKE4EMySHsgCI%3D&amp;x-signature-webp=67RReRXh9gVLQilAmQ7kP%2BxyQUk%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/33b107e073684cc6ac77dba9bccf5f02~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=FWuaDeD06ey%2B8F6YDBiTxqsWcfg%3D&amp;x-signature-webp=lxRiyFhNXO%2BICWZ3C%2BXe02DE3iM%3D</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -8889,12 +10694,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=JJDsqmXPE785hYKZRffQtEi1x2k%3D&amp;x-signature-webp=JUneY87LJqx%2BfdAPeNPx65dblGA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=KxW%2FEv%2FZPm5Tr6qsPRsaR8Hwd3o%3D&amp;x-signature-webp=X0pf3N4Ke%2BpPNRNy7mLKTp4Snh8%3D</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=LP2RXdVUoq%2BcoZmcSzUhowZOzaA%3D&amp;x-signature-webp=R5fCCsBxUZKklWU6U9bpyECi6co%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e140811d00c343c3b00983a8d73258b2~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=KxW%2FEv%2FZPm5Tr6qsPRsaR8Hwd3o%3D&amp;x-signature-webp=X0pf3N4Ke%2BpPNRNy7mLKTp4Snh8%3D</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -8939,12 +10744,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=iUujNWD9UkeWfjC69b6x%2BCe1eEk%3D&amp;x-signature-webp=U1COq%2F0RkmE%2F4r0NJz6ymhy7BtU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=Z63dV%2BXuCj8ot1r1nJULWKqHUxg%3D&amp;x-signature-webp=ZOE2nrBkGzz8Pd81yQUSW4HGoxw%3D</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=iUujNWD9UkeWfjC69b6x%2BCe1eEk%3D&amp;x-signature-webp=U1COq%2F0RkmE%2F4r0NJz6ymhy7BtU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9b0225eaec684b00915445a816ff3992~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=Z63dV%2BXuCj8ot1r1nJULWKqHUxg%3D&amp;x-signature-webp=ZOE2nrBkGzz8Pd81yQUSW4HGoxw%3D</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -8989,12 +10794,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=TZexh%2F1rHRKlwQX8vs5uyLZZSjk%3D&amp;x-signature-webp=v5ofvoUUvnl%2Bnj36PaO3CpfSQJc%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=avYJt9P47i7tQfeYBx3wb2qPwTw%3D&amp;x-signature-webp=gw6fCLHQeNrvT%2FtnjWPjbUsjnYY%3D</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604341&amp;x-signature=TZexh%2F1rHRKlwQX8vs5uyLZZSjk%3D&amp;x-signature-webp=v5ofvoUUvnl%2Bnj36PaO3CpfSQJc%3D</t>
+          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1bad1d2dc25c44f88797cc5dad2f220e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646017&amp;x-signature=CCwseyuN2FYDF31u1DnZCyylCEU%3D&amp;x-signature-webp=ILRW8ogGwz1elXh6vVuTaxJtVtU%3D</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -9204,12 +11009,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=%2FFwwqWaNvZdwruwp%2BNJw%2BKF%2FuFs%3D&amp;x-signature-webp=AnZBI%2FTNDFGO9U8ZQixt6v%2B509A%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=UHRS3L9fCzWRI5Mv8TgaUHFfO3E%3D&amp;x-signature-webp=jJ9GvtcNqj70tc60O1kw89b32%2Bw%3D</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=bnjkc%2BoLG%2B4REoJUm3DdHWDfu6Q%3D&amp;x-signature-webp=5KoB4oRbA9UJrdoplKPyy6OlbgY%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/36e962fa59734122a5c603bd3b617457~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=gHqhcnS6p%2BFNCzziLIIfyOl25tk%3D&amp;x-signature-webp=HueiNA6W%2BqwRjAoSTkBBfrCHupE%3D</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -9254,12 +11059,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=wVnXi7THp5FtYJHyCRGrcOGx%2BFE%3D&amp;x-signature-webp=uSyuCSgr0q5cjstt9qa8ahm83PE%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=lZeu7C6aK4bjBLGWFDddFFeg%2BFE%3D&amp;x-signature-webp=gix3sHTEbgot1YYcvt94uit46iI%3D</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=MT3hw4t%2FRWIhxL5dbrIRKmxxn5o%3D&amp;x-signature-webp=UBQcXpYQ2niWyHcTYl4ED%2B01s6M%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/81a7fb788e4146f5b2340e5a7c7c43f7~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=tptzOnKDpn1qlSol8WWNc%2BtLJeQ%3D&amp;x-signature-webp=j79tiZbAxWjcuEbh9Pi3ckRxhlg%3D</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -9304,12 +11109,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=5R6bzPRXu2Py7FmejIIhIoFdnHw%3D&amp;x-signature-webp=wczkX6X%2F6xnpAqx1oGOT1c8eDVw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=Bw6teuiMfsmK8NMVjTyt1GTactg%3D&amp;x-signature-webp=0LskqGPE25qB4cwFNGQRqhZ6taw%3D</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=4cKukYWdWR%2FRWPngrshbUQ6bGZY%3D&amp;x-signature-webp=4oDmGX%2FeVnyMdB6PjX5qbOeyeQA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/632c63c42ca44b858f25d82ec9d7ce60~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=%2FpxhlUIDgHLrdUoPhTb80MddJQk%3D&amp;x-signature-webp=SY6xaaV0cPff5ClKDv6aRA82TdU%3D</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -9354,12 +11159,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=6jxF%2B2%2FXpDO4pcoiX11r2pPSeuM%3D&amp;x-signature-webp=psK1x639Vjsc7E5Xi7nxIEh0oTQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=EbWMLrqpMLGpORahKe1%2BLiUMzpQ%3D&amp;x-signature-webp=BOUrY8Dpq2ukJK3Gv3IRSrvaY6w%3D</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=ZKWCupCGNMkZVHwAK4YVmEsf5%2FI%3D&amp;x-signature-webp=afQEjkIHY%2BsY2sDwS8KNSCMqvlc%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5bb6e96ad0374e8bbaf0f13fd15e4534~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=qyHW%2F4o0zWMNo6jHTbk4vuCHgug%3D&amp;x-signature-webp=PjYDDq9DwzrdzkZYYIYJWZA2004%3D</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -9404,12 +11209,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=W3p2zPMK6d1mP5UHL4mOm3VD3aE%3D&amp;x-signature-webp=EntRhQ7rBqgEkexcjjvef8S1PsE%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=cUuAAydx2LaOua2pACovM4Niidc%3D&amp;x-signature-webp=B4Qu18bZe0QvxPAVUNzVpLn2oGw%3D</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=W3p2zPMK6d1mP5UHL4mOm3VD3aE%3D&amp;x-signature-webp=EntRhQ7rBqgEkexcjjvef8S1PsE%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/66488a928e8042519c6676d816cd6471~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=cUuAAydx2LaOua2pACovM4Niidc%3D&amp;x-signature-webp=B4Qu18bZe0QvxPAVUNzVpLn2oGw%3D</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -9454,12 +11259,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=GTwlZXJxHoplnnkSDJ13D6QSVK8%3D&amp;x-signature-webp=yBj%2BGD9d43khH29f5rZQz%2Blf8VM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=XmHZ2xT17HsceQ6arKyjq0e27cU%3D&amp;x-signature-webp=pzPaLXx6iWy2%2BbM1mwe4LrZI5wc%3D</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604345&amp;x-signature=GTwlZXJxHoplnnkSDJ13D6QSVK8%3D&amp;x-signature-webp=yBj%2BGD9d43khH29f5rZQz%2Blf8VM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1754b3fc687d4f4b9dfdc746f39386bc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646020&amp;x-signature=XmHZ2xT17HsceQ6arKyjq0e27cU%3D&amp;x-signature-webp=pzPaLXx6iWy2%2BbM1mwe4LrZI5wc%3D</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -9614,12 +11419,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2B%2FqDYKSQU2iQY82D%2F04kwKtDrnA%3D&amp;x-signature-webp=U1W4UNKcuFeFrxUyFXoAk49zVdU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=Tbv3SzY4pEdpnKY%2F%2FAHiLk2OUxo%3D&amp;x-signature-webp=x6%2FYKs%2B1jqrgT0fxT6dete4Neio%3D</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=PfXPLLP21IYKhrtFym%2FKy%2F67amM%3D&amp;x-signature-webp=sG5sDRdrHsBKiPVaJdKXU2pijFU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/805d27da245d458883c5089b8f2cf1fc~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=ra4rDzB8tdjNj3S8kkgRDc9O2gY%3D&amp;x-signature-webp=i8veO8QbB4xsbHTQ3JQmaV6EkoE%3D</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -9664,12 +11469,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=PjEZtnYONb0GEoAfAIH4BEKa1lg%3D&amp;x-signature-webp=V6drDG7x0MudqCYfWkb5FTBs6SM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=NCgs4BPRULa9SVHE4XymMNM6gQ8%3D&amp;x-signature-webp=ck0EXTnn44e4OyL8z%2BZTYVixgHs%3D</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2BcCz0hnqjwm9xfeqMf08dtOg4SQ%3D&amp;x-signature-webp=jK%2FVOETyeBCyZ1SYyB192pMwf1o%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/d43539d7a5384fcebdc259d5f206ccc8~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=pfQt8YIJKjoLSDVf5eSzr80vVuA%3D&amp;x-signature-webp=WY%2FwXU%2Fi4zf4sAwk62a2zlbyyV0%3D</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -9714,12 +11519,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=vEP1H1e%2FcdMFuq6I4S5Y%2B5JzSto%3D&amp;x-signature-webp=N1e4aj2k8HcihssYPJ477K%2BVwzA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=BMPKDGFuGiYnf6Ka%2FNYc8%2BZ5l9E%3D&amp;x-signature-webp=C1Tj%2FldGi9dN9a%2FVhgBRmIoNEBg%3D</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=OH%2FUrYAchBU14UcHePdZcnjIGvE%3D&amp;x-signature-webp=OudiBBwO3cHJQ%2BTiKwb%2FfQAiZJA%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1ef728ec8f8b4f74a86d3869e1ce1f27~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=rRd8KXj9db%2BfiucesbMTt4TjVW4%3D&amp;x-signature-webp=pMXSRCkhhGndBWgVR1JzsCllbn8%3D</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -9764,12 +11569,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=0IuXjlHYaijpntTooGIdKoTJ474%3D&amp;x-signature-webp=M8En%2B13b4itIZiYzrQ8K4oI9HzQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=71x%2F%2BHY0Gc%2FMvDt0EcH4yMNk5T4%3D&amp;x-signature-webp=uY926%2FVTfX5Itg4rOIdR%2BVQIpIM%3D</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=QQzoTzNlMP06FcRS%2BNjwnFxgkFs%3D&amp;x-signature-webp=HxYShILalfMGRgSzvtE%2FA5W23cQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/4b21de2dd1b44f93a8cc4bd0b8760f22~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=bz8srJuLOjiCYDeXsF1BGMSEPio%3D&amp;x-signature-webp=LcrIKwTOASxwTvluPAZBkkCRGtU%3D</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -9814,12 +11619,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=fpdtfLXoP6mS9U40r9oRGv8vuc0%3D&amp;x-signature-webp=YfGeB%2Byz4krOJda%2BG0Bs2QWH6Os%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=RBB33UQkJouuV3trfY8ZLAVEM4E%3D&amp;x-signature-webp=YPYb3jSntbW%2BK1PDNNPxVfTw4ww%3D</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=BYaBpIkp4O22mSTGhHvbcYNgDlU%3D&amp;x-signature-webp=VYhzprLxRhvFGhcCPS9B4VRCY4M%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/b45228aee24a42d296d6784e0de8ad60~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=WpZ%2F3hiEKvDcdNlYsl6vOtH1yL0%3D&amp;x-signature-webp=O4Ujnv9Z0gODmNnu%2Fd4Kv5%2BaAk0%3D</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -9864,12 +11669,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=%2Bl1f32hH99dRDOxN%2B7XO2Hxry5k%3D&amp;x-signature-webp=MhmyDPKb1%2BrlA7ZX9lMVU3eqFJg%3D</t>
+          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=4qN%2B2zzlw72Ly%2BzwEIvAp3X1nt0%3D&amp;x-signature-webp=JyNfnN3CzJgWJGn2c3EejbVQzgU%3D</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=EcxCYNm7mVDrxwrbny8OJLcf9Yc%3D&amp;x-signature-webp=I491YAsSy0ZZ1oMazcJVyTeA9W8%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3a97d8cff33f4afab7a92750c6ea97bd~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=5buFaNVA5StU8IU4NvN5ljoDnQU%3D&amp;x-signature-webp=WtWuYOkcOUrjAktxkf7ZhC8atC4%3D</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -9914,12 +11719,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=TyjJGpuCkRBmLsxJNKhmzePzXig%3D&amp;x-signature-webp=wgoxJaBlU6nC2l%2BI0F1dsFGh7zI%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=pz36nJZN%2FLELk8U5vRHRYeifCu8%3D&amp;x-signature-webp=wBbAZHUdxRT8lKa%2B4eVlOC9q6Z4%3D</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=mp%2FNPx%2FJeSAGs%2B8AlQRhH1pQiuk%3D&amp;x-signature-webp=i4BCAglcGhJK%2FqwEVlJxCo9%2BLFM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/282694eb40374192b9e194c520c91b0d~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=NQqLZkxdaPma1jV15PgmLChLmjQ%3D&amp;x-signature-webp=mZAcV3cSgRtYmMhEeR1ZLsxoj6A%3D</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -9964,12 +11769,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=awJdlSl%2F1GQjHweRRXzILjHL1JI%3D&amp;x-signature-webp=ZI19cOWc%2FCtz4YnEnd2hOzYzJ0c%3D</t>
+          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=HtpS%2BJcNmXMU3cLWQorpBDxNA%2Bc%3D&amp;x-signature-webp=%2BcrXy0adH1s6DDunjvNXQtHo6V8%3D</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=TZ8LPgWji8hwWc%2BJGDwLujVzunk%3D&amp;x-signature-webp=Pi%2B94l3rJOJEOp%2FJmOE1vTQHVUw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/5806fc2a7e6c448b87838e59e75f1929~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=8oGT6tz4UBMwmFyMsaoe9zfXTvg%3D&amp;x-signature-webp=UZHoufb6ZSpO%2Ff0OLyODLmG6b40%3D</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -10014,12 +11819,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=IPDcC%2Bg9IvVN708HG%2BlFs1HbqnU%3D&amp;x-signature-webp=kAJoLffigibljWjZ3gdDqmqngzw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=s3XpZJFXR2zBwZizMgnLKyrYWNw%3D&amp;x-signature-webp=IUbEhRgmlsIqC7y3F4eFSYZ0HMo%3D</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=IPDcC%2Bg9IvVN708HG%2BlFs1HbqnU%3D&amp;x-signature-webp=kAJoLffigibljWjZ3gdDqmqngzw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/01c44a71ca8d4f43999a6e8fa94f0724~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=s3XpZJFXR2zBwZizMgnLKyrYWNw%3D&amp;x-signature-webp=IUbEhRgmlsIqC7y3F4eFSYZ0HMo%3D</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -10064,12 +11869,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=8MfAkc9zYs6C%2FiIBhPx3BpPJwsw%3D&amp;x-signature-webp=sCCJZWYd%2BEy79PXHgHq0UInRviw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=P1WWhj4g85KoTql%2BIF1uywv7ef0%3D&amp;x-signature-webp=UBhM50sYzZWs%2F0KGoN%2FyAWCboQY%3D</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=8MfAkc9zYs6C%2FiIBhPx3BpPJwsw%3D&amp;x-signature-webp=sCCJZWYd%2BEy79PXHgHq0UInRviw%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/17559de5f5f846daa12442c61d6f21c9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=P1WWhj4g85KoTql%2BIF1uywv7ef0%3D&amp;x-signature-webp=UBhM50sYzZWs%2F0KGoN%2FyAWCboQY%3D</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -10114,12 +11919,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=BsdT094hOEdEVVoPIK0dtvIzIGg%3D&amp;x-signature-webp=P6979aJFlO5Wvbg5T5Tfq4t8eF0%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=bS0uKvQG9446EsvLtwNd6dwIBsI%3D&amp;x-signature-webp=41X68TO8cz8oodz8gu5TIW088T4%3D</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=BsdT094hOEdEVVoPIK0dtvIzIGg%3D&amp;x-signature-webp=P6979aJFlO5Wvbg5T5Tfq4t8eF0%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/1e5c62974cfe4f06848cd22418272c87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=bS0uKvQG9446EsvLtwNd6dwIBsI%3D&amp;x-signature-webp=41X68TO8cz8oodz8gu5TIW088T4%3D</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -10164,12 +11969,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=rrUT5pVf05k8KerYH%2FilR0OnPH0%3D&amp;x-signature-webp=RTMh%2F%2BMnt%2Ff%2BCxf0DA3DzZ4ReLg%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=5sKpH73qCtr7ic7Tsob7iE1gpPM%3D&amp;x-signature-webp=6jzUOQ5ggjoEeD7P8glx4kZ%2F0ac%3D</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604349&amp;x-signature=rrUT5pVf05k8KerYH%2FilR0OnPH0%3D&amp;x-signature-webp=RTMh%2F%2BMnt%2Ff%2BCxf0DA3DzZ4ReLg%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3de569aff3154f90840bf0a9ecfb4ff9~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646024&amp;x-signature=5sKpH73qCtr7ic7Tsob7iE1gpPM%3D&amp;x-signature-webp=6jzUOQ5ggjoEeD7P8glx4kZ%2F0ac%3D</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -10489,12 +12294,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=t%2BLknu0CWcUWk13YnZIIHDJOl6U%3D&amp;x-signature-webp=XDg%2B6AwCrmhFMLEce4DQOs3Inmk%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Efci3BJtcP1Nh8%2F41pcOhqiXuIE%3D&amp;x-signature-webp=YMLls2p9Rh%2B8LkdlWOHSZPfXazk%3D</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=5gPP9gPPhQwkXDA8PJycGqzRQKU%3D&amp;x-signature-webp=hgiaDyukCNwpldMVNzBC5G5ltQs%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f2998fb257e94aa18a47108f1861705e~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=ZHQud5OUyQ0tC%2FX2znNkTSJNCgU%3D&amp;x-signature-webp=apAnKal4TRUTPymTB3qoRYpdcYg%3D</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -10539,12 +12344,12 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=PE9y%2BTMK3jdlhFzrfu2YpWI1I%2FQ%3D&amp;x-signature-webp=rXQG8RhZQfjCwwNbJ6yXGeD%2Fsj4%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Dkf9Gkw4AxdKLRM0Xj4U%2FDJ9HOY%3D&amp;x-signature-webp=PeyEebN5r1EI9Ivoz14wZs3F1v0%3D</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=2FGALqS7QZAEFEQ9zBiKX9joQkE%3D&amp;x-signature-webp=Dk8I4zVrV%2FeH1aIVL8o8XSW5cyI%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/e40ad8327867413a91371d97d5907a87~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=08cpJpJPLTsnk6PR6fa9j31LiT0%3D&amp;x-signature-webp=4I7G4XxKAj%2BOngkmgCgtZ6Vbdqw%3D</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -10589,12 +12394,12 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=7xj5hESN8V2BmNlbxzQRgxWcICQ%3D&amp;x-signature-webp=MtcaHaC%2FZ0yNQJ1r2EpctEn1Qko%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=Xd2mVZHSwsaoWFzptDfGC3JldGQ%3D&amp;x-signature-webp=zKd5ebneXXRuS9qC1lztMv9kpzU%3D</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604353&amp;x-signature=0aG1CCSh3QMWlI0jrPZ%2BzCnyz%2Bo%3D&amp;x-signature-webp=LfDT3VbA8O0VE0Nfn6uGFQOlUZM%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/6b23678b76a348f5ad2c9cb33895723a~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646029&amp;x-signature=eJIEjgaevccbNj1MmPpBD8z4E%2BU%3D&amp;x-signature-webp=OV5TvXV%2FIshatB2UZC55ZkYl81M%3D</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -10749,12 +12554,12 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=WI%2BmGBMcNKHVwFjKOlIuXlvfYCs%3D&amp;x-signature-webp=WdUTi75634FjssOYBX5fYA13RgQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=JzuGZkBT%2FivUuAES754e3G7xEBg%3D&amp;x-signature-webp=qU1UVGZCXDI2%2FoUWU2Wr2VrWYtg%3D</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=MK6fJJVIbP6aRahiJ3ZkDRqmrRc%3D&amp;x-signature-webp=vdu%2Fnm9Jzbimt4fd%2BJtRUCbhwao%3D</t>
+          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/f459dd5b748e424e9c656220f3bc9b12~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=KI5Kwe8G4ici%2Bp5BgU3Bl7FJbdU%3D&amp;x-signature-webp=3Ml8X0qYxScVSxfp6et%2BrO%2Faesw%3D</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -10799,12 +12604,12 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=8p3LU9ULew1tA6kHyThPuUY%2BCK0%3D&amp;x-signature-webp=VnZqmwhR8zB5P2OrF0HPj1c83uo%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=0oAWPPB9%2FWirKROikDeV7UqZ%2BjY%3D&amp;x-signature-webp=J%2FTOGC%2BcIaDazz1DbxQKh8HTZGo%3D</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=YzFqNgXx%2FaS3gDVeol7j5DNp2Uk%3D&amp;x-signature-webp=QQfxvD%2FCBvCQ86nHqBq75rnSMBI%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/9aa346acb295436d948b9cb50e68fddf~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=iv5PQpfP2qzCtRkKF2OlYZyfzVo%3D&amp;x-signature-webp=2rYMAK4psrhLMgEv2q8FdkeQHdE%3D</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -10849,12 +12654,12 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=7D4Zbq9RA7TAxtuczetEF04Nyj0%3D&amp;x-signature-webp=nmeBl5FzXCci8wbiEqZKvSENJfI%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=96AAJ2Sx9khmvt2Pc2vksX4Nbjk%3D&amp;x-signature-webp=Pbx0bxSLhIfoYM2cPbQH%2Fkaeg5c%3D</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=kW0wQdIsL31dh0B1QPZ8U0q6%2FQE%3D&amp;x-signature-webp=tH6M5t%2FGCp4rZRFiQNE32RPxOMQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/ef3c8764dce0463d953d434d342e945b~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=PJS77AA%2BDjw7QNaxLvmcD1gugcc%3D&amp;x-signature-webp=29Q4DVwmS%2BOgc2TgxKbFf1XnUuE%3D</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -10899,12 +12704,12 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=AiQYogKrI3ZKM7OCLoF7mF%2BXt3M%3D&amp;x-signature-webp=%2BH9Si15hpZah3hrDCUrMfB1igdg%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=6HKct0z0vV8o6rt0dlS97YnX4rM%3D&amp;x-signature-webp=J%2B10JMv9SYpOR5szhoCfH8wd3Tk%3D</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=HpLU7ZSEqWYnetBuPuMMMWX5uPQ%3D&amp;x-signature-webp=2XSvzUPQE%2BJEhLRk%2BDBcWHobtNU%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3ac71c0a7062435c887a1060946f4d00~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=zEnoWcNjLnovk8FIrMb7RXquMxE%3D&amp;x-signature-webp=b38JgVWEdPAA8VA62%2Ff9V9RdaVM%3D</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -10949,12 +12754,12 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>https://p19-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=ZU0AiqbegW%2BpfBRTg3wvrmQ3a5M%3D&amp;x-signature-webp=dara6IKBD2z7%2BEwfHNKwsHdqtOc%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:700:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=zxq4qogcgI2kpsBJOUDVUmnBhVc%3D&amp;x-signature-webp=JQRRUOHHKFymUqK%2F1ajq7QEDUiM%3D</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789604364&amp;x-signature=Jj45yr%2FTckz63D6c8UKKJ8m3EXo%3D&amp;x-signature-webp=A%2F6ERR2dj5nOk4X4pXmxWbBF%2FKQ%3D</t>
+          <t>https://p16-images-sign-sg.tokopedia-static.net/tos-alisg-i-aphluv4xwc-sg/3c173fb0e65b48c2afbeca2c0ab0392d~tplv-aphluv4xwc-resize-jpeg:200:0.jpeg?lk3s=0ccea506&amp;x-expires=1789646031&amp;x-signature=5toO3Gt6HGwIPCF2gdIb24kUZNE%3D&amp;x-signature-webp=i1eXu%2BvLMNRCFoW8SQeQmpL%2BPyc%3D</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -11606,13 +13411,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11651,7 +13456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-17T04:18:44+07:00</t>
+          <t>2026-09-17T15:53:00+07:00</t>
         </is>
       </c>
     </row>
@@ -11663,7 +13468,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17T04:20:09+07:00</t>
+          <t>2026-09-17T15:54:22+07:00</t>
         </is>
       </c>
     </row>
@@ -11730,64 +13535,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>media_rows</t>
+          <t>detail_rows</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>74</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>images_downloaded</t>
+          <t>products_with_detail</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>74</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>images_directory</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>C:\Portfolio\Niuva_Tokopedia_Scraper_v2.1_All_JPG\niuva_v21\Niuva_Product_Images</t>
-        </is>
+          <t>media_rows</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>image_format</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>jpg</t>
-        </is>
+          <t>images_downloaded</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>jpeg_quality</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>95</v>
+          <t>images_directory</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C:\Portfolio\Niuva_Tokopedia_Scraper_v2.1_All_JPG\niuva_v21\Niuva_Product_Images</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>image_format</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>jpeg_quality</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Data comes from public Tokopedia pages. Fields can be empty if unavailable or if page structures change.</t>
         </is>
@@ -11798,7 +13623,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>